<commit_message>
data: cierre dia 2026-09-13_1434 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DFC5FE34-825F-4C20-A4E0-3433DE441431}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4FCFD03D-9EE4-4ECE-BD5E-20EBC45724FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -572,7 +572,8 @@
     <col min="4" max="4" width="16" customWidth="1"/>
     <col min="5" max="7" width="25" customWidth="1"/>
     <col min="8" max="8" width="15" customWidth="1"/>
-    <col min="9" max="11" width="13" customWidth="1"/>
+    <col min="9" max="10" width="13" customWidth="1"/>
+    <col min="11" max="11" width="14" customWidth="1"/>
     <col min="12" max="13" width="12" customWidth="1"/>
     <col min="14" max="14" width="16" customWidth="1"/>
     <col min="15" max="15" width="14" customWidth="1"/>
@@ -665,22 +666,22 @@
         <v>0</v>
       </c>
       <c r="K2">
-        <v>5639071.9199999999</v>
+        <v>5126429.0199999996</v>
       </c>
       <c r="L2">
-        <v>64.97</v>
+        <v>59.06</v>
       </c>
       <c r="M2">
-        <v>225562.88</v>
+        <v>205057.16</v>
       </c>
       <c r="N2">
-        <v>428291.42</v>
+        <v>458883.66</v>
       </c>
       <c r="O2">
-        <v>73717.86</v>
+        <v>0</v>
       </c>
       <c r="P2">
-        <v>49027.62</v>
+        <v>0</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -712,28 +713,28 @@
         <v>61320000</v>
       </c>
       <c r="I3">
-        <v>21461811.100000001</v>
+        <v>21583909.280000001</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>53654527.759999998</v>
+        <v>49054339.270000003</v>
       </c>
       <c r="L3">
-        <v>87.5</v>
+        <v>80</v>
       </c>
       <c r="M3">
-        <v>2146181.11</v>
+        <v>1962173.57</v>
       </c>
       <c r="N3">
-        <v>2657212.59</v>
+        <v>2838292.19</v>
       </c>
       <c r="O3">
-        <v>0</v>
+        <v>1246182.58</v>
       </c>
       <c r="P3">
-        <v>6482530.5899999999</v>
+        <v>2419878.06</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -765,28 +766,28 @@
         <v>130000000</v>
       </c>
       <c r="I4">
-        <v>57835761.200000003</v>
+        <v>79320757.269999996</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>144589403</v>
+        <v>180274448.34</v>
       </c>
       <c r="L4">
-        <v>111.22</v>
+        <v>138.66999999999999</v>
       </c>
       <c r="M4">
-        <v>5783576.1200000001</v>
+        <v>7210977.9299999997</v>
       </c>
       <c r="N4">
-        <v>4810949.25</v>
+        <v>3619945.91</v>
       </c>
       <c r="O4">
-        <v>303709.89</v>
+        <v>8386588.4299999997</v>
       </c>
       <c r="P4">
-        <v>0</v>
+        <v>10429780.050000001</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -824,22 +825,22 @@
         <v>0</v>
       </c>
       <c r="K5">
-        <v>5570818.9800000004</v>
+        <v>5064380.8899999997</v>
       </c>
       <c r="L5">
-        <v>57.14</v>
+        <v>51.94</v>
       </c>
       <c r="M5">
-        <v>222832.76</v>
+        <v>202575.24</v>
       </c>
       <c r="N5">
-        <v>501444.83</v>
+        <v>537262.31000000006</v>
       </c>
       <c r="O5">
-        <v>28074.79</v>
+        <v>0</v>
       </c>
       <c r="P5">
-        <v>0</v>
+        <v>389041.16</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -877,22 +878,22 @@
         <v>0</v>
       </c>
       <c r="K6">
-        <v>22790177.550000001</v>
+        <v>20718343.219999999</v>
       </c>
       <c r="L6">
-        <v>70.12</v>
+        <v>63.75</v>
       </c>
       <c r="M6">
-        <v>911607.1</v>
+        <v>828733.73</v>
       </c>
       <c r="N6">
-        <v>1558928.6</v>
+        <v>1670280.64</v>
       </c>
       <c r="O6">
-        <v>22110.77</v>
+        <v>145665.26</v>
       </c>
       <c r="P6">
-        <v>0</v>
+        <v>329124.67</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -924,28 +925,28 @@
         <v>113750000</v>
       </c>
       <c r="I7">
-        <v>10307300.060000001</v>
+        <v>10460954.619999999</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>25768250.149999999</v>
+        <v>23774896.870000001</v>
       </c>
       <c r="L7">
-        <v>22.65</v>
+        <v>20.9</v>
       </c>
       <c r="M7">
-        <v>1030730.01</v>
+        <v>950995.87</v>
       </c>
       <c r="N7">
-        <v>6896180</v>
+        <v>7377788.96</v>
       </c>
       <c r="O7">
-        <v>2214418.16</v>
+        <v>766591.77</v>
       </c>
       <c r="P7">
-        <v>535067.81000000006</v>
+        <v>242815.89</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -983,22 +984,22 @@
         <v>0</v>
       </c>
       <c r="K8">
-        <v>19990977.649999999</v>
+        <v>18173616.039999999</v>
       </c>
       <c r="L8">
-        <v>51.26</v>
+        <v>46.6</v>
       </c>
       <c r="M8">
-        <v>799639.11</v>
+        <v>726944.64</v>
       </c>
       <c r="N8">
-        <v>2066907.26</v>
+        <v>2214543.5</v>
       </c>
       <c r="O8">
-        <v>0</v>
+        <v>-57681.64</v>
       </c>
       <c r="P8">
-        <v>0</v>
+        <v>519079.97</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1076,7 +1077,7 @@
         <v>40</v>
       </c>
       <c r="H2">
-        <v>1.6</v>
+        <v>2.2000000000000002</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1232,7 +1233,7 @@
         <v>40</v>
       </c>
       <c r="H8">
-        <v>22.6</v>
+        <v>22.3</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -1258,7 +1259,7 @@
         <v>42</v>
       </c>
       <c r="H9">
-        <v>1.8</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
data: cierre dia 2026-09-14_1718 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4FCFD03D-9EE4-4ECE-BD5E-20EBC45724FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{10CC9C39-D049-4EC8-8ED0-1907EFE8872E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -666,22 +666,22 @@
         <v>0</v>
       </c>
       <c r="K2">
-        <v>5126429.0199999996</v>
+        <v>4699226.5999999996</v>
       </c>
       <c r="L2">
-        <v>59.06</v>
+        <v>54.14</v>
       </c>
       <c r="M2">
-        <v>205057.16</v>
+        <v>187969.06</v>
       </c>
       <c r="N2">
-        <v>458883.66</v>
+        <v>494182.40000000002</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>40005.5</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -713,28 +713,28 @@
         <v>61320000</v>
       </c>
       <c r="I3">
-        <v>21583909.280000001</v>
+        <v>22137186.620000001</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>49054339.270000003</v>
+        <v>46119138.789999999</v>
       </c>
       <c r="L3">
-        <v>80</v>
+        <v>75.209999999999994</v>
       </c>
       <c r="M3">
-        <v>1962173.57</v>
+        <v>1844765.55</v>
       </c>
       <c r="N3">
-        <v>2838292.19</v>
+        <v>3014062.57</v>
       </c>
       <c r="O3">
-        <v>1246182.58</v>
+        <v>1063684.73</v>
       </c>
       <c r="P3">
-        <v>2419878.06</v>
+        <v>5163141.7699999996</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -766,28 +766,28 @@
         <v>130000000</v>
       </c>
       <c r="I4">
-        <v>79320757.269999996</v>
+        <v>91691672.319999993</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>180274448.34</v>
+        <v>191024317.33000001</v>
       </c>
       <c r="L4">
-        <v>138.66999999999999</v>
+        <v>146.94</v>
       </c>
       <c r="M4">
-        <v>7210977.9299999997</v>
+        <v>7640972.6900000004</v>
       </c>
       <c r="N4">
-        <v>3619945.91</v>
+        <v>2946794.44</v>
       </c>
       <c r="O4">
-        <v>8386588.4299999997</v>
+        <v>1613072.09</v>
       </c>
       <c r="P4">
-        <v>10429780.050000001</v>
+        <v>2218349.9</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -825,22 +825,22 @@
         <v>0</v>
       </c>
       <c r="K5">
-        <v>5064380.8899999997</v>
+        <v>4642349.1500000004</v>
       </c>
       <c r="L5">
-        <v>51.94</v>
+        <v>47.61</v>
       </c>
       <c r="M5">
-        <v>202575.24</v>
+        <v>185693.97</v>
       </c>
       <c r="N5">
-        <v>537262.31000000006</v>
+        <v>578590.18999999994</v>
       </c>
       <c r="O5">
         <v>0</v>
       </c>
       <c r="P5">
-        <v>389041.16</v>
+        <v>21094.7</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -872,28 +872,28 @@
         <v>32500000</v>
       </c>
       <c r="I6">
-        <v>9116071.0199999996</v>
+        <v>9279962.1500000004</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>20718343.219999999</v>
+        <v>19333254.469999999</v>
       </c>
       <c r="L6">
-        <v>63.75</v>
+        <v>59.49</v>
       </c>
       <c r="M6">
-        <v>828733.73</v>
+        <v>773330.18</v>
       </c>
       <c r="N6">
-        <v>1670280.64</v>
+        <v>1786156.76</v>
       </c>
       <c r="O6">
-        <v>145665.26</v>
+        <v>137793.60000000001</v>
       </c>
       <c r="P6">
-        <v>329124.67</v>
+        <v>4297326.75</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -925,28 +925,28 @@
         <v>113750000</v>
       </c>
       <c r="I7">
-        <v>10460954.619999999</v>
+        <v>10904755.310000001</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>23774896.870000001</v>
+        <v>22718240.23</v>
       </c>
       <c r="L7">
-        <v>20.9</v>
+        <v>19.97</v>
       </c>
       <c r="M7">
-        <v>950995.87</v>
+        <v>908729.61</v>
       </c>
       <c r="N7">
-        <v>7377788.96</v>
+        <v>7911172.6699999999</v>
       </c>
       <c r="O7">
-        <v>766591.77</v>
+        <v>592826.14</v>
       </c>
       <c r="P7">
-        <v>242815.89</v>
+        <v>658011.37</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -978,28 +978,28 @@
         <v>39000000</v>
       </c>
       <c r="I8">
-        <v>7996391.0599999996</v>
+        <v>9970804.6699999999</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>18173616.039999999</v>
+        <v>20772509.73</v>
       </c>
       <c r="L8">
-        <v>46.6</v>
+        <v>53.26</v>
       </c>
       <c r="M8">
-        <v>726944.64</v>
+        <v>830900.39</v>
       </c>
       <c r="N8">
-        <v>2214543.5</v>
+        <v>2233015.0299999998</v>
       </c>
       <c r="O8">
-        <v>-57681.64</v>
+        <v>398859.56</v>
       </c>
       <c r="P8">
-        <v>519079.97</v>
+        <v>407749.33</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1077,7 +1077,7 @@
         <v>40</v>
       </c>
       <c r="H2">
-        <v>2.2000000000000002</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1103,7 +1103,7 @@
         <v>40</v>
       </c>
       <c r="H3">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1129,7 +1129,7 @@
         <v>40</v>
       </c>
       <c r="H4">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1155,7 +1155,7 @@
         <v>40</v>
       </c>
       <c r="H5">
-        <v>0</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -1233,7 +1233,7 @@
         <v>40</v>
       </c>
       <c r="H8">
-        <v>22.3</v>
+        <v>21.4</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -1259,7 +1259,7 @@
         <v>42</v>
       </c>
       <c r="H9">
-        <v>1.7</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -1285,7 +1285,7 @@
         <v>42</v>
       </c>
       <c r="H10">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: cierre dia 2026-09-15_1718 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{10CC9C39-D049-4EC8-8ED0-1907EFE8872E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{04F0A1D2-BFA2-4EEA-8FE7-18E51EC6DFEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -666,22 +666,22 @@
         <v>0</v>
       </c>
       <c r="K2">
-        <v>4699226.5999999996</v>
+        <v>4337747.63</v>
       </c>
       <c r="L2">
-        <v>54.14</v>
+        <v>49.97</v>
       </c>
       <c r="M2">
-        <v>187969.06</v>
+        <v>173509.91</v>
       </c>
       <c r="N2">
-        <v>494182.40000000002</v>
+        <v>535364.27</v>
       </c>
       <c r="O2">
-        <v>0</v>
+        <v>1670796.73</v>
       </c>
       <c r="P2">
-        <v>40005.5</v>
+        <v>-2846.54</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -713,28 +713,28 @@
         <v>61320000</v>
       </c>
       <c r="I3">
-        <v>22137186.620000001</v>
+        <v>23820903.77</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>46119138.789999999</v>
+        <v>45809430.32</v>
       </c>
       <c r="L3">
-        <v>75.209999999999994</v>
+        <v>74.709999999999994</v>
       </c>
       <c r="M3">
-        <v>1844765.55</v>
+        <v>1832377.21</v>
       </c>
       <c r="N3">
-        <v>3014062.57</v>
+        <v>3124924.69</v>
       </c>
       <c r="O3">
-        <v>1063684.73</v>
+        <v>1731426.1</v>
       </c>
       <c r="P3">
-        <v>5163141.7699999996</v>
+        <v>251569.42</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -766,28 +766,28 @@
         <v>130000000</v>
       </c>
       <c r="I4">
-        <v>91691672.319999993</v>
+        <v>91711970.739999995</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>191024317.33000001</v>
+        <v>176369174.50999999</v>
       </c>
       <c r="L4">
-        <v>146.94</v>
+        <v>135.66999999999999</v>
       </c>
       <c r="M4">
-        <v>7640972.6900000004</v>
+        <v>7054766.9800000004</v>
       </c>
       <c r="N4">
-        <v>2946794.44</v>
+        <v>3190669.1</v>
       </c>
       <c r="O4">
-        <v>1613072.09</v>
+        <v>671706.69</v>
       </c>
       <c r="P4">
-        <v>2218349.9</v>
+        <v>1681446.15</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -825,22 +825,22 @@
         <v>0</v>
       </c>
       <c r="K5">
-        <v>4642349.1500000004</v>
+        <v>4285245.37</v>
       </c>
       <c r="L5">
-        <v>47.61</v>
+        <v>43.95</v>
       </c>
       <c r="M5">
-        <v>185693.97</v>
+        <v>171409.81</v>
       </c>
       <c r="N5">
-        <v>578590.18999999994</v>
+        <v>626806.03</v>
       </c>
       <c r="O5">
         <v>0</v>
       </c>
       <c r="P5">
-        <v>21094.7</v>
+        <v>285080.27</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -872,28 +872,28 @@
         <v>32500000</v>
       </c>
       <c r="I6">
-        <v>9279962.1500000004</v>
+        <v>9611363.4000000004</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>19333254.469999999</v>
+        <v>18483391.16</v>
       </c>
       <c r="L6">
-        <v>59.49</v>
+        <v>56.87</v>
       </c>
       <c r="M6">
-        <v>773330.18</v>
+        <v>739335.65</v>
       </c>
       <c r="N6">
-        <v>1786156.76</v>
+        <v>1907386.38</v>
       </c>
       <c r="O6">
-        <v>137793.60000000001</v>
+        <v>396666.79</v>
       </c>
       <c r="P6">
-        <v>4297326.75</v>
+        <v>457101.09</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -925,28 +925,28 @@
         <v>113750000</v>
       </c>
       <c r="I7">
-        <v>10904755.310000001</v>
+        <v>14315081.140000001</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>22718240.23</v>
+        <v>27529002.190000001</v>
       </c>
       <c r="L7">
-        <v>19.97</v>
+        <v>24.2</v>
       </c>
       <c r="M7">
-        <v>908729.61</v>
+        <v>1101160.0900000001</v>
       </c>
       <c r="N7">
-        <v>7911172.6699999999</v>
+        <v>8286243.2400000002</v>
       </c>
       <c r="O7">
-        <v>592826.14</v>
+        <v>297833.75</v>
       </c>
       <c r="P7">
-        <v>658011.37</v>
+        <v>404109.01</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -978,28 +978,28 @@
         <v>39000000</v>
       </c>
       <c r="I8">
-        <v>9970804.6699999999</v>
+        <v>10136211.51</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>20772509.73</v>
+        <v>19492714.440000001</v>
       </c>
       <c r="L8">
-        <v>53.26</v>
+        <v>49.98</v>
       </c>
       <c r="M8">
-        <v>830900.39</v>
+        <v>779708.58</v>
       </c>
       <c r="N8">
-        <v>2233015.0299999998</v>
+        <v>2405315.71</v>
       </c>
       <c r="O8">
-        <v>398859.56</v>
+        <v>568183.43000000005</v>
       </c>
       <c r="P8">
-        <v>407749.33</v>
+        <v>219976.32000000001</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1077,7 +1077,7 @@
         <v>40</v>
       </c>
       <c r="H2">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1103,7 +1103,7 @@
         <v>40</v>
       </c>
       <c r="H3">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1129,7 +1129,7 @@
         <v>40</v>
       </c>
       <c r="H4">
-        <v>0.8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1233,7 +1233,7 @@
         <v>40</v>
       </c>
       <c r="H8">
-        <v>21.4</v>
+        <v>16.5</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
data: cierre dia 2026-09-16_1901 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{04F0A1D2-BFA2-4EEA-8FE7-18E51EC6DFEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A9EB91DD-2EB9-49B5-B138-055C2AE66A79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -666,22 +666,22 @@
         <v>0</v>
       </c>
       <c r="K2">
-        <v>4337747.63</v>
+        <v>4027908.51</v>
       </c>
       <c r="L2">
-        <v>49.97</v>
+        <v>46.4</v>
       </c>
       <c r="M2">
-        <v>173509.91</v>
+        <v>161116.34</v>
       </c>
       <c r="N2">
-        <v>535364.27</v>
+        <v>584033.75</v>
       </c>
       <c r="O2">
-        <v>1670796.73</v>
+        <v>32339.59</v>
       </c>
       <c r="P2">
-        <v>-2846.54</v>
+        <v>418008.11</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -713,28 +713,28 @@
         <v>61320000</v>
       </c>
       <c r="I3">
-        <v>23820903.77</v>
+        <v>24267351.440000001</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>45809430.32</v>
+        <v>43334556.130000003</v>
       </c>
       <c r="L3">
-        <v>74.709999999999994</v>
+        <v>70.67</v>
       </c>
       <c r="M3">
-        <v>1832377.21</v>
+        <v>1733382.25</v>
       </c>
       <c r="N3">
-        <v>3124924.69</v>
+        <v>3368422.6</v>
       </c>
       <c r="O3">
-        <v>1731426.1</v>
+        <v>153860.60999999999</v>
       </c>
       <c r="P3">
-        <v>251569.42</v>
+        <v>2220714.69</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -766,28 +766,28 @@
         <v>130000000</v>
       </c>
       <c r="I4">
-        <v>91711970.739999995</v>
+        <v>94088032.870000005</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>176369174.50999999</v>
+        <v>168014344.41999999</v>
       </c>
       <c r="L4">
-        <v>135.66999999999999</v>
+        <v>129.24</v>
       </c>
       <c r="M4">
-        <v>7054766.9800000004</v>
+        <v>6720573.7800000003</v>
       </c>
       <c r="N4">
-        <v>3190669.1</v>
+        <v>3264724.28</v>
       </c>
       <c r="O4">
-        <v>671706.69</v>
+        <v>28036566.23</v>
       </c>
       <c r="P4">
-        <v>1681446.15</v>
+        <v>627271.53</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -819,28 +819,28 @@
         <v>9750000</v>
       </c>
       <c r="I5">
-        <v>2228327.59</v>
+        <v>2536683.13</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>4285245.37</v>
+        <v>4529791.3</v>
       </c>
       <c r="L5">
-        <v>43.95</v>
+        <v>46.46</v>
       </c>
       <c r="M5">
-        <v>171409.81</v>
+        <v>181191.65</v>
       </c>
       <c r="N5">
-        <v>626806.03</v>
+        <v>655756.07999999996</v>
       </c>
       <c r="O5">
-        <v>0</v>
+        <v>49468.89</v>
       </c>
       <c r="P5">
-        <v>285080.27</v>
+        <v>0</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -872,28 +872,28 @@
         <v>32500000</v>
       </c>
       <c r="I6">
-        <v>9611363.4000000004</v>
+        <v>9931240.1199999992</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>18483391.16</v>
+        <v>17734357.359999999</v>
       </c>
       <c r="L6">
-        <v>56.87</v>
+        <v>54.57</v>
       </c>
       <c r="M6">
-        <v>739335.65</v>
+        <v>709374.29</v>
       </c>
       <c r="N6">
-        <v>1907386.38</v>
+        <v>2051705.44</v>
       </c>
       <c r="O6">
-        <v>396666.79</v>
+        <v>1183017.07</v>
       </c>
       <c r="P6">
-        <v>457101.09</v>
+        <v>92082.79</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -925,28 +925,28 @@
         <v>113750000</v>
       </c>
       <c r="I7">
-        <v>14315081.140000001</v>
+        <v>14785249.75</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>27529002.190000001</v>
+        <v>26402231.690000001</v>
       </c>
       <c r="L7">
-        <v>24.2</v>
+        <v>23.21</v>
       </c>
       <c r="M7">
-        <v>1101160.0900000001</v>
+        <v>1056089.27</v>
       </c>
       <c r="N7">
-        <v>8286243.2400000002</v>
+        <v>8996795.4800000004</v>
       </c>
       <c r="O7">
-        <v>297833.75</v>
+        <v>1994036.11</v>
       </c>
       <c r="P7">
-        <v>404109.01</v>
+        <v>559130.48</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -978,28 +978,28 @@
         <v>39000000</v>
       </c>
       <c r="I8">
-        <v>10136211.51</v>
+        <v>12780838.02</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>19492714.440000001</v>
+        <v>22822925.039999999</v>
       </c>
       <c r="L8">
-        <v>49.98</v>
+        <v>58.52</v>
       </c>
       <c r="M8">
-        <v>779708.58</v>
+        <v>912917</v>
       </c>
       <c r="N8">
-        <v>2405315.71</v>
+        <v>2383560.1800000002</v>
       </c>
       <c r="O8">
-        <v>568183.43000000005</v>
+        <v>1910602.8</v>
       </c>
       <c r="P8">
-        <v>219976.32000000001</v>
+        <v>169926.52</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1077,7 +1077,7 @@
         <v>40</v>
       </c>
       <c r="H2">
-        <v>1.8</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1207,7 +1207,7 @@
         <v>40</v>
       </c>
       <c r="H7">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -1233,7 +1233,7 @@
         <v>40</v>
       </c>
       <c r="H8">
-        <v>16.5</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -1259,7 +1259,7 @@
         <v>42</v>
       </c>
       <c r="H9">
-        <v>1.5</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
data: cierre dia 2026-09-17_1753 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A9EB91DD-2EB9-49B5-B138-055C2AE66A79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{AFCE341C-7B2F-4E52-B5AC-2E6BE2573645}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -660,28 +660,28 @@
         <v>8680000</v>
       </c>
       <c r="I2">
-        <v>2255628.77</v>
+        <v>2801831.16</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>4027908.51</v>
+        <v>4669718.59</v>
       </c>
       <c r="L2">
-        <v>46.4</v>
+        <v>53.8</v>
       </c>
       <c r="M2">
-        <v>161116.34</v>
+        <v>186788.74</v>
       </c>
       <c r="N2">
-        <v>584033.75</v>
+        <v>587816.88</v>
       </c>
       <c r="O2">
-        <v>32339.59</v>
+        <v>-25420.1</v>
       </c>
       <c r="P2">
-        <v>418008.11</v>
+        <v>0</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -713,28 +713,28 @@
         <v>61320000</v>
       </c>
       <c r="I3">
-        <v>24267351.440000001</v>
+        <v>38372015.520000003</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>43334556.130000003</v>
+        <v>63953359.210000001</v>
       </c>
       <c r="L3">
-        <v>70.67</v>
+        <v>104.29</v>
       </c>
       <c r="M3">
-        <v>1733382.25</v>
+        <v>2558134.37</v>
       </c>
       <c r="N3">
-        <v>3368422.6</v>
+        <v>2294798.4500000002</v>
       </c>
       <c r="O3">
-        <v>153860.60999999999</v>
+        <v>326830.42</v>
       </c>
       <c r="P3">
-        <v>2220714.69</v>
+        <v>343979.88</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -766,28 +766,28 @@
         <v>130000000</v>
       </c>
       <c r="I4">
-        <v>94088032.870000005</v>
+        <v>94868069.989999995</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>168014344.41999999</v>
+        <v>158113449.99000001</v>
       </c>
       <c r="L4">
-        <v>129.24</v>
+        <v>121.63</v>
       </c>
       <c r="M4">
-        <v>6720573.7800000003</v>
+        <v>6324538</v>
       </c>
       <c r="N4">
-        <v>3264724.28</v>
+        <v>3513193</v>
       </c>
       <c r="O4">
-        <v>28036566.23</v>
+        <v>2343794.06</v>
       </c>
       <c r="P4">
-        <v>627271.53</v>
+        <v>1335695.71</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -819,28 +819,28 @@
         <v>9750000</v>
       </c>
       <c r="I5">
-        <v>2536683.13</v>
+        <v>2593073.7999999998</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>4529791.3</v>
+        <v>4321789.67</v>
       </c>
       <c r="L5">
-        <v>46.46</v>
+        <v>44.33</v>
       </c>
       <c r="M5">
-        <v>181191.65</v>
+        <v>172871.59</v>
       </c>
       <c r="N5">
-        <v>655756.07999999996</v>
+        <v>715692.62</v>
       </c>
       <c r="O5">
-        <v>49468.89</v>
+        <v>1776305.96</v>
       </c>
       <c r="P5">
-        <v>0</v>
+        <v>68302.98</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -872,28 +872,28 @@
         <v>32500000</v>
       </c>
       <c r="I6">
-        <v>9931240.1199999992</v>
+        <v>10306471.039999999</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>17734357.359999999</v>
+        <v>17177451.739999998</v>
       </c>
       <c r="L6">
-        <v>54.57</v>
+        <v>52.85</v>
       </c>
       <c r="M6">
-        <v>709374.29</v>
+        <v>687098.07</v>
       </c>
       <c r="N6">
-        <v>2051705.44</v>
+        <v>2219352.9</v>
       </c>
       <c r="O6">
-        <v>1183017.07</v>
+        <v>2100481.14</v>
       </c>
       <c r="P6">
-        <v>92082.79</v>
+        <v>127705.67</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -925,28 +925,28 @@
         <v>113750000</v>
       </c>
       <c r="I7">
-        <v>14785249.75</v>
+        <v>15258448.720000001</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>26402231.690000001</v>
+        <v>25430747.870000001</v>
       </c>
       <c r="L7">
-        <v>23.21</v>
+        <v>22.36</v>
       </c>
       <c r="M7">
-        <v>1056089.27</v>
+        <v>1017229.91</v>
       </c>
       <c r="N7">
-        <v>8996795.4800000004</v>
+        <v>9849155.1300000008</v>
       </c>
       <c r="O7">
-        <v>1994036.11</v>
+        <v>641164.41</v>
       </c>
       <c r="P7">
-        <v>559130.48</v>
+        <v>708960.31</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -978,28 +978,28 @@
         <v>39000000</v>
       </c>
       <c r="I8">
-        <v>12780838.02</v>
+        <v>14335457.85</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>22822925.039999999</v>
+        <v>23892429.75</v>
       </c>
       <c r="L8">
-        <v>58.52</v>
+        <v>61.26</v>
       </c>
       <c r="M8">
-        <v>912917</v>
+        <v>955697.19</v>
       </c>
       <c r="N8">
-        <v>2383560.1800000002</v>
+        <v>2466454.2200000002</v>
       </c>
       <c r="O8">
-        <v>1910602.8</v>
+        <v>3571862.36</v>
       </c>
       <c r="P8">
-        <v>169926.52</v>
+        <v>463032.88</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1077,7 +1077,7 @@
         <v>40</v>
       </c>
       <c r="H2">
-        <v>1.7</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1103,7 +1103,7 @@
         <v>40</v>
       </c>
       <c r="H3">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1129,7 +1129,7 @@
         <v>40</v>
       </c>
       <c r="H4">
-        <v>1</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1155,7 +1155,7 @@
         <v>40</v>
       </c>
       <c r="H5">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -1181,7 +1181,7 @@
         <v>40</v>
       </c>
       <c r="H6">
-        <v>2.6</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -1233,7 +1233,7 @@
         <v>40</v>
       </c>
       <c r="H8">
-        <v>16</v>
+        <v>15.5</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -1285,7 +1285,7 @@
         <v>42</v>
       </c>
       <c r="H10">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: cierre dia 2026-09-18_1745 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AFCE341C-7B2F-4E52-B5AC-2E6BE2573645}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{399E0C5B-4BA3-4459-BBD2-15BFB2C5884A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -660,28 +660,28 @@
         <v>8680000</v>
       </c>
       <c r="I2">
-        <v>2801831.16</v>
+        <v>2757582.92</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>4669718.59</v>
+        <v>4308723.32</v>
       </c>
       <c r="L2">
-        <v>53.8</v>
+        <v>49.64</v>
       </c>
       <c r="M2">
-        <v>186788.74</v>
+        <v>172348.93</v>
       </c>
       <c r="N2">
-        <v>587816.88</v>
+        <v>658046.34</v>
       </c>
       <c r="O2">
-        <v>-25420.1</v>
+        <v>0</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>73717.86</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -713,28 +713,28 @@
         <v>61320000</v>
       </c>
       <c r="I3">
-        <v>38372015.520000003</v>
+        <v>38937652.619999997</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>63953359.210000001</v>
+        <v>60840082.210000001</v>
       </c>
       <c r="L3">
-        <v>104.29</v>
+        <v>99.22</v>
       </c>
       <c r="M3">
-        <v>2558134.37</v>
+        <v>2433603.29</v>
       </c>
       <c r="N3">
-        <v>2294798.4500000002</v>
+        <v>2486927.4900000002</v>
       </c>
       <c r="O3">
-        <v>326830.42</v>
+        <v>122098.18</v>
       </c>
       <c r="P3">
-        <v>343979.88</v>
+        <v>0</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -766,28 +766,28 @@
         <v>130000000</v>
       </c>
       <c r="I4">
-        <v>94868069.989999995</v>
+        <v>95249128.519999996</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>158113449.99000001</v>
+        <v>148826763.31</v>
       </c>
       <c r="L4">
-        <v>121.63</v>
+        <v>114.48</v>
       </c>
       <c r="M4">
-        <v>6324538</v>
+        <v>5953070.5300000003</v>
       </c>
       <c r="N4">
-        <v>3513193</v>
+        <v>3861207.94</v>
       </c>
       <c r="O4">
-        <v>2343794.06</v>
+        <v>21346389.219999999</v>
       </c>
       <c r="P4">
-        <v>1335695.71</v>
+        <v>303709.89</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -825,22 +825,22 @@
         <v>0</v>
       </c>
       <c r="K5">
-        <v>4321789.67</v>
+        <v>4051677.81</v>
       </c>
       <c r="L5">
-        <v>44.33</v>
+        <v>41.56</v>
       </c>
       <c r="M5">
-        <v>172871.59</v>
+        <v>162067.10999999999</v>
       </c>
       <c r="N5">
-        <v>715692.62</v>
+        <v>795214.02</v>
       </c>
       <c r="O5">
-        <v>1776305.96</v>
+        <v>0</v>
       </c>
       <c r="P5">
-        <v>68302.98</v>
+        <v>28074.79</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -872,28 +872,28 @@
         <v>32500000</v>
       </c>
       <c r="I6">
-        <v>10306471.039999999</v>
+        <v>10453369.17</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>17177451.739999998</v>
+        <v>16333389.32</v>
       </c>
       <c r="L6">
-        <v>52.85</v>
+        <v>50.26</v>
       </c>
       <c r="M6">
-        <v>687098.07</v>
+        <v>653335.56999999995</v>
       </c>
       <c r="N6">
-        <v>2219352.9</v>
+        <v>2449625.65</v>
       </c>
       <c r="O6">
-        <v>2100481.14</v>
+        <v>0</v>
       </c>
       <c r="P6">
-        <v>127705.67</v>
+        <v>22110.77</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -925,28 +925,28 @@
         <v>113750000</v>
       </c>
       <c r="I7">
-        <v>15258448.720000001</v>
+        <v>16017010.210000001</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>25430747.870000001</v>
+        <v>25026578.449999999</v>
       </c>
       <c r="L7">
-        <v>22.36</v>
+        <v>22</v>
       </c>
       <c r="M7">
-        <v>1017229.91</v>
+        <v>1001063.14</v>
       </c>
       <c r="N7">
-        <v>9849155.1300000008</v>
+        <v>10859221.09</v>
       </c>
       <c r="O7">
-        <v>641164.41</v>
+        <v>153654.56</v>
       </c>
       <c r="P7">
-        <v>708960.31</v>
+        <v>2214418.16</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -978,28 +978,28 @@
         <v>39000000</v>
       </c>
       <c r="I8">
-        <v>14335457.85</v>
+        <v>14527966.91</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>23892429.75</v>
+        <v>22699948.289999999</v>
       </c>
       <c r="L8">
-        <v>61.26</v>
+        <v>58.2</v>
       </c>
       <c r="M8">
-        <v>955697.19</v>
+        <v>907997.93</v>
       </c>
       <c r="N8">
-        <v>2466454.2200000002</v>
+        <v>2719114.79</v>
       </c>
       <c r="O8">
-        <v>3571862.36</v>
+        <v>0</v>
       </c>
       <c r="P8">
-        <v>463032.88</v>
+        <v>0</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1077,7 +1077,7 @@
         <v>40</v>
       </c>
       <c r="H2">
-        <v>1.5</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1103,7 +1103,7 @@
         <v>40</v>
       </c>
       <c r="H3">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1129,7 +1129,7 @@
         <v>40</v>
       </c>
       <c r="H4">
-        <v>1.5</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1155,7 +1155,7 @@
         <v>40</v>
       </c>
       <c r="H5">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -1233,7 +1233,7 @@
         <v>40</v>
       </c>
       <c r="H8">
-        <v>15.5</v>
+        <v>14.8</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -1285,7 +1285,7 @@
         <v>42</v>
       </c>
       <c r="H10">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: cierre dia 2026-09-20_1134 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{399E0C5B-4BA3-4459-BBD2-15BFB2C5884A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F85E738C-F088-4940-94E7-CF1E8BF1A23A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -660,28 +660,28 @@
         <v>8680000</v>
       </c>
       <c r="I2">
-        <v>2757582.92</v>
+        <v>2813508.45</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>4308723.32</v>
+        <v>3907650.63</v>
       </c>
       <c r="L2">
-        <v>49.64</v>
+        <v>45.02</v>
       </c>
       <c r="M2">
-        <v>172348.93</v>
+        <v>156306.03</v>
       </c>
       <c r="N2">
-        <v>658046.34</v>
+        <v>838070.22</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2">
-        <v>73717.86</v>
+        <v>0</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -713,28 +713,28 @@
         <v>61320000</v>
       </c>
       <c r="I3">
-        <v>38937652.619999997</v>
+        <v>45420183.210000001</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>60840082.210000001</v>
+        <v>63083587.789999999</v>
       </c>
       <c r="L3">
-        <v>99.22</v>
+        <v>102.88</v>
       </c>
       <c r="M3">
-        <v>2433603.29</v>
+        <v>2523343.5099999998</v>
       </c>
       <c r="N3">
-        <v>2486927.4900000002</v>
+        <v>2271402.4</v>
       </c>
       <c r="O3">
-        <v>122098.18</v>
+        <v>531485.19999999995</v>
       </c>
       <c r="P3">
-        <v>0</v>
+        <v>1246182.58</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -772,22 +772,22 @@
         <v>0</v>
       </c>
       <c r="K4">
-        <v>148826763.31</v>
+        <v>132290456.27</v>
       </c>
       <c r="L4">
-        <v>114.48</v>
+        <v>101.76</v>
       </c>
       <c r="M4">
-        <v>5953070.5300000003</v>
+        <v>5291618.25</v>
       </c>
       <c r="N4">
-        <v>3861207.94</v>
+        <v>4964410.21</v>
       </c>
       <c r="O4">
-        <v>21346389.219999999</v>
+        <v>12360675.48</v>
       </c>
       <c r="P4">
-        <v>303709.89</v>
+        <v>8386588.4299999997</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -825,22 +825,22 @@
         <v>0</v>
       </c>
       <c r="K5">
-        <v>4051677.81</v>
+        <v>3601491.39</v>
       </c>
       <c r="L5">
-        <v>41.56</v>
+        <v>36.94</v>
       </c>
       <c r="M5">
-        <v>162067.10999999999</v>
+        <v>144059.66</v>
       </c>
       <c r="N5">
-        <v>795214.02</v>
+        <v>1022418.03</v>
       </c>
       <c r="O5">
         <v>0</v>
       </c>
       <c r="P5">
-        <v>28074.79</v>
+        <v>0</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -878,22 +878,22 @@
         <v>0</v>
       </c>
       <c r="K6">
-        <v>16333389.32</v>
+        <v>14518568.289999999</v>
       </c>
       <c r="L6">
-        <v>50.26</v>
+        <v>44.67</v>
       </c>
       <c r="M6">
-        <v>653335.56999999995</v>
+        <v>580742.73</v>
       </c>
       <c r="N6">
-        <v>2449625.65</v>
+        <v>3149518.69</v>
       </c>
       <c r="O6">
-        <v>0</v>
+        <v>163891.13</v>
       </c>
       <c r="P6">
-        <v>22110.77</v>
+        <v>145665.26</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -925,28 +925,28 @@
         <v>113750000</v>
       </c>
       <c r="I7">
-        <v>16017010.210000001</v>
+        <v>20945317.370000001</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>25026578.449999999</v>
+        <v>29090718.57</v>
       </c>
       <c r="L7">
-        <v>22</v>
+        <v>25.57</v>
       </c>
       <c r="M7">
-        <v>1001063.14</v>
+        <v>1163628.74</v>
       </c>
       <c r="N7">
-        <v>10859221.09</v>
+        <v>13257811.800000001</v>
       </c>
       <c r="O7">
-        <v>153654.56</v>
+        <v>443800.69</v>
       </c>
       <c r="P7">
-        <v>2214418.16</v>
+        <v>766591.77</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -978,28 +978,28 @@
         <v>39000000</v>
       </c>
       <c r="I8">
-        <v>14527966.91</v>
+        <v>14498429.390000001</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>22699948.289999999</v>
+        <v>20136707.48</v>
       </c>
       <c r="L8">
-        <v>58.2</v>
+        <v>51.63</v>
       </c>
       <c r="M8">
-        <v>907997.93</v>
+        <v>805468.3</v>
       </c>
       <c r="N8">
-        <v>2719114.79</v>
+        <v>3500224.37</v>
       </c>
       <c r="O8">
-        <v>0</v>
+        <v>1974413.61</v>
       </c>
       <c r="P8">
-        <v>0</v>
+        <v>-57681.64</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1077,7 +1077,7 @@
         <v>40</v>
       </c>
       <c r="H2">
-        <v>1.4</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1103,7 +1103,7 @@
         <v>40</v>
       </c>
       <c r="H3">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1155,7 +1155,7 @@
         <v>40</v>
       </c>
       <c r="H5">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -1233,7 +1233,7 @@
         <v>40</v>
       </c>
       <c r="H8">
-        <v>14.8</v>
+        <v>11.4</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -1285,7 +1285,7 @@
         <v>42</v>
       </c>
       <c r="H10">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: cierre dia 2026-09-21_1714 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F85E738C-F088-4940-94E7-CF1E8BF1A23A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B92EC4DC-8CF2-4ACB-B259-2289DE343ACB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -572,7 +572,8 @@
     <col min="4" max="4" width="16" customWidth="1"/>
     <col min="5" max="7" width="25" customWidth="1"/>
     <col min="8" max="8" width="15" customWidth="1"/>
-    <col min="9" max="10" width="13" customWidth="1"/>
+    <col min="9" max="9" width="14" customWidth="1"/>
+    <col min="10" max="10" width="13" customWidth="1"/>
     <col min="11" max="11" width="14" customWidth="1"/>
     <col min="12" max="13" width="12" customWidth="1"/>
     <col min="14" max="14" width="16" customWidth="1"/>
@@ -713,28 +714,28 @@
         <v>61320000</v>
       </c>
       <c r="I3">
-        <v>45420183.210000001</v>
+        <v>46044416.969999999</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>63083587.789999999</v>
+        <v>63950579.130000003</v>
       </c>
       <c r="L3">
-        <v>102.88</v>
+        <v>104.29</v>
       </c>
       <c r="M3">
-        <v>2523343.5099999998</v>
+        <v>2558023.17</v>
       </c>
       <c r="N3">
-        <v>2271402.4</v>
+        <v>2182226.15</v>
       </c>
       <c r="O3">
-        <v>531485.19999999995</v>
+        <v>1670173.09</v>
       </c>
       <c r="P3">
-        <v>1246182.58</v>
+        <v>1063684.73</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -766,28 +767,28 @@
         <v>130000000</v>
       </c>
       <c r="I4">
-        <v>95249128.519999996</v>
+        <v>109262025.56</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>132290456.27</v>
+        <v>151752813.28</v>
       </c>
       <c r="L4">
-        <v>101.76</v>
+        <v>116.73</v>
       </c>
       <c r="M4">
-        <v>5291618.25</v>
+        <v>6070112.5300000003</v>
       </c>
       <c r="N4">
-        <v>4964410.21</v>
+        <v>2962567.78</v>
       </c>
       <c r="O4">
-        <v>12360675.48</v>
+        <v>97710.18</v>
       </c>
       <c r="P4">
-        <v>8386588.4299999997</v>
+        <v>1613072.09</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -872,28 +873,28 @@
         <v>32500000</v>
       </c>
       <c r="I6">
-        <v>10453369.17</v>
+        <v>10623611.27</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>14518568.289999999</v>
+        <v>14755015.65</v>
       </c>
       <c r="L6">
-        <v>44.67</v>
+        <v>45.4</v>
       </c>
       <c r="M6">
-        <v>580742.73</v>
+        <v>590200.63</v>
       </c>
       <c r="N6">
-        <v>3149518.69</v>
+        <v>3125198.39</v>
       </c>
       <c r="O6">
-        <v>163891.13</v>
+        <v>331401.26</v>
       </c>
       <c r="P6">
-        <v>145665.26</v>
+        <v>137793.60000000001</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -925,28 +926,28 @@
         <v>113750000</v>
       </c>
       <c r="I7">
-        <v>20945317.370000001</v>
+        <v>21584241.52</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>29090718.57</v>
+        <v>29978113.219999999</v>
       </c>
       <c r="L7">
-        <v>25.57</v>
+        <v>26.35</v>
       </c>
       <c r="M7">
-        <v>1163628.74</v>
+        <v>1199124.53</v>
       </c>
       <c r="N7">
-        <v>13257811.800000001</v>
+        <v>13166536.93</v>
       </c>
       <c r="O7">
-        <v>443800.69</v>
+        <v>3390840.82</v>
       </c>
       <c r="P7">
-        <v>766591.77</v>
+        <v>592826.14</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -978,28 +979,28 @@
         <v>39000000</v>
       </c>
       <c r="I8">
-        <v>14498429.390000001</v>
+        <v>24551147.57</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>20136707.48</v>
+        <v>34098816.07</v>
       </c>
       <c r="L8">
-        <v>51.63</v>
+        <v>87.43</v>
       </c>
       <c r="M8">
-        <v>805468.3</v>
+        <v>1363952.6399999999</v>
       </c>
       <c r="N8">
-        <v>3500224.37</v>
+        <v>2064121.78</v>
       </c>
       <c r="O8">
-        <v>1974413.61</v>
+        <v>165406.84</v>
       </c>
       <c r="P8">
-        <v>-57681.64</v>
+        <v>398859.56</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1077,7 +1078,7 @@
         <v>40</v>
       </c>
       <c r="H2">
-        <v>1.7</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1129,7 +1130,7 @@
         <v>40</v>
       </c>
       <c r="H4">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1207,7 +1208,7 @@
         <v>40</v>
       </c>
       <c r="H7">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -1233,7 +1234,7 @@
         <v>40</v>
       </c>
       <c r="H8">
-        <v>11.4</v>
+        <v>11.6</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -1259,7 +1260,7 @@
         <v>42</v>
       </c>
       <c r="H9">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
data: cierre dia 2026-09-23_0745 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B92EC4DC-8CF2-4ACB-B259-2289DE343ACB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F31EBC26-1312-40F8-B066-14D8CF04F4D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -573,8 +573,7 @@
     <col min="5" max="7" width="25" customWidth="1"/>
     <col min="8" max="8" width="15" customWidth="1"/>
     <col min="9" max="9" width="14" customWidth="1"/>
-    <col min="10" max="10" width="13" customWidth="1"/>
-    <col min="11" max="11" width="14" customWidth="1"/>
+    <col min="10" max="11" width="13" customWidth="1"/>
     <col min="12" max="13" width="12" customWidth="1"/>
     <col min="14" max="14" width="16" customWidth="1"/>
     <col min="15" max="15" width="14" customWidth="1"/>
@@ -667,22 +666,22 @@
         <v>0</v>
       </c>
       <c r="K2">
-        <v>3907650.63</v>
+        <v>3701984.8</v>
       </c>
       <c r="L2">
-        <v>45.02</v>
+        <v>42.65</v>
       </c>
       <c r="M2">
-        <v>156306.03</v>
+        <v>148079.39000000001</v>
       </c>
       <c r="N2">
-        <v>838070.22</v>
+        <v>977748.59</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>1670796.73</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -714,28 +713,28 @@
         <v>61320000</v>
       </c>
       <c r="I3">
-        <v>46044416.969999999</v>
+        <v>47642079.049999997</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>63950579.130000003</v>
+        <v>62686946.119999997</v>
       </c>
       <c r="L3">
-        <v>104.29</v>
+        <v>102.23</v>
       </c>
       <c r="M3">
-        <v>2558023.17</v>
+        <v>2507477.84</v>
       </c>
       <c r="N3">
-        <v>2182226.15</v>
+        <v>2279653.4900000002</v>
       </c>
       <c r="O3">
-        <v>1670173.09</v>
+        <v>481783.87</v>
       </c>
       <c r="P3">
-        <v>1063684.73</v>
+        <v>1731426.1</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -767,28 +766,28 @@
         <v>130000000</v>
       </c>
       <c r="I4">
-        <v>109262025.56</v>
+        <v>111648934.15000001</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>151752813.28</v>
+        <v>146906492.30000001</v>
       </c>
       <c r="L4">
-        <v>116.73</v>
+        <v>113</v>
       </c>
       <c r="M4">
-        <v>6070112.5300000003</v>
+        <v>5876259.6900000004</v>
       </c>
       <c r="N4">
-        <v>2962567.78</v>
+        <v>3058510.98</v>
       </c>
       <c r="O4">
-        <v>97710.18</v>
+        <v>2250370.58</v>
       </c>
       <c r="P4">
-        <v>1613072.09</v>
+        <v>671706.69</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -820,25 +819,25 @@
         <v>9750000</v>
       </c>
       <c r="I5">
-        <v>2593073.7999999998</v>
+        <v>4990657.7300000004</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>3601491.39</v>
+        <v>6566654.9100000001</v>
       </c>
       <c r="L5">
-        <v>36.94</v>
+        <v>67.349999999999994</v>
       </c>
       <c r="M5">
-        <v>144059.66</v>
+        <v>262666.2</v>
       </c>
       <c r="N5">
-        <v>1022418.03</v>
+        <v>793223.71</v>
       </c>
       <c r="O5">
-        <v>0</v>
+        <v>308355.53999999998</v>
       </c>
       <c r="P5">
         <v>0</v>
@@ -873,28 +872,28 @@
         <v>32500000</v>
       </c>
       <c r="I6">
-        <v>10623611.27</v>
+        <v>13023181.460000001</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>14755015.65</v>
+        <v>17135765.079999998</v>
       </c>
       <c r="L6">
-        <v>45.4</v>
+        <v>52.73</v>
       </c>
       <c r="M6">
-        <v>590200.63</v>
+        <v>685430.6</v>
       </c>
       <c r="N6">
-        <v>3125198.39</v>
+        <v>3246136.42</v>
       </c>
       <c r="O6">
-        <v>331401.26</v>
+        <v>319876.71999999997</v>
       </c>
       <c r="P6">
-        <v>137793.60000000001</v>
+        <v>396666.79</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -926,28 +925,28 @@
         <v>113750000</v>
       </c>
       <c r="I7">
-        <v>21584241.52</v>
+        <v>24724519.300000001</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>29978113.219999999</v>
+        <v>32532262.239999998</v>
       </c>
       <c r="L7">
-        <v>26.35</v>
+        <v>28.6</v>
       </c>
       <c r="M7">
-        <v>1199124.53</v>
+        <v>1301290.49</v>
       </c>
       <c r="N7">
-        <v>13166536.93</v>
+        <v>14837580.119999999</v>
       </c>
       <c r="O7">
-        <v>3390840.82</v>
+        <v>489653.62</v>
       </c>
       <c r="P7">
-        <v>592826.14</v>
+        <v>297833.75</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -979,28 +978,28 @@
         <v>39000000</v>
       </c>
       <c r="I8">
-        <v>24551147.57</v>
+        <v>27721316.34</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>34098816.07</v>
+        <v>36475416.229999997</v>
       </c>
       <c r="L8">
-        <v>87.43</v>
+        <v>93.53</v>
       </c>
       <c r="M8">
-        <v>1363952.6399999999</v>
+        <v>1459016.65</v>
       </c>
       <c r="N8">
-        <v>2064121.78</v>
+        <v>1879780.61</v>
       </c>
       <c r="O8">
-        <v>165406.84</v>
+        <v>2644626.5099999998</v>
       </c>
       <c r="P8">
-        <v>398859.56</v>
+        <v>568183.43000000005</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1078,7 +1077,7 @@
         <v>40</v>
       </c>
       <c r="H2">
-        <v>1.3</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1130,7 +1129,7 @@
         <v>40</v>
       </c>
       <c r="H4">
-        <v>1.3</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1156,7 +1155,7 @@
         <v>40</v>
       </c>
       <c r="H5">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -1234,7 +1233,7 @@
         <v>40</v>
       </c>
       <c r="H8">
-        <v>11.6</v>
+        <v>10.4</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -1286,7 +1285,7 @@
         <v>42</v>
       </c>
       <c r="H10">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: cierre dia 2026-09-23_1748 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F31EBC26-1312-40F8-B066-14D8CF04F4D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E3468A4E-9AB3-4419-BB58-3881DCD8280B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -573,7 +573,8 @@
     <col min="5" max="7" width="25" customWidth="1"/>
     <col min="8" max="8" width="15" customWidth="1"/>
     <col min="9" max="9" width="14" customWidth="1"/>
-    <col min="10" max="11" width="13" customWidth="1"/>
+    <col min="10" max="10" width="13" customWidth="1"/>
+    <col min="11" max="11" width="14" customWidth="1"/>
     <col min="12" max="13" width="12" customWidth="1"/>
     <col min="14" max="14" width="16" customWidth="1"/>
     <col min="15" max="15" width="14" customWidth="1"/>
@@ -666,22 +667,22 @@
         <v>0</v>
       </c>
       <c r="K2">
-        <v>3701984.8</v>
+        <v>3516885.56</v>
       </c>
       <c r="L2">
-        <v>42.65</v>
+        <v>40.520000000000003</v>
       </c>
       <c r="M2">
-        <v>148079.39000000001</v>
+        <v>140675.42000000001</v>
       </c>
       <c r="N2">
-        <v>977748.59</v>
+        <v>1173298.31</v>
       </c>
       <c r="O2">
-        <v>0</v>
+        <v>501954.16</v>
       </c>
       <c r="P2">
-        <v>1670796.73</v>
+        <v>32339.59</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -713,28 +714,28 @@
         <v>61320000</v>
       </c>
       <c r="I3">
-        <v>47642079.049999997</v>
+        <v>60274602.219999999</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>62686946.119999997</v>
+        <v>75343252.769999996</v>
       </c>
       <c r="L3">
-        <v>102.23</v>
+        <v>122.87</v>
       </c>
       <c r="M3">
-        <v>2507477.84</v>
+        <v>3013730.11</v>
       </c>
       <c r="N3">
-        <v>2279653.4900000002</v>
+        <v>209079.56</v>
       </c>
       <c r="O3">
-        <v>481783.87</v>
+        <v>14104664.09</v>
       </c>
       <c r="P3">
-        <v>1731426.1</v>
+        <v>153860.60999999999</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -766,28 +767,28 @@
         <v>130000000</v>
       </c>
       <c r="I4">
-        <v>111648934.15000001</v>
+        <v>127386291.16</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>146906492.30000001</v>
+        <v>159232863.94999999</v>
       </c>
       <c r="L4">
-        <v>113</v>
+        <v>122.49</v>
       </c>
       <c r="M4">
-        <v>5876259.6900000004</v>
+        <v>6369314.5599999996</v>
       </c>
       <c r="N4">
-        <v>3058510.98</v>
+        <v>522741.77</v>
       </c>
       <c r="O4">
-        <v>2250370.58</v>
+        <v>1017675.24</v>
       </c>
       <c r="P4">
-        <v>671706.69</v>
+        <v>27847207.91</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -819,28 +820,28 @@
         <v>9750000</v>
       </c>
       <c r="I5">
-        <v>4990657.7300000004</v>
+        <v>5096126.7300000004</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>6566654.9100000001</v>
+        <v>6370158.4100000001</v>
       </c>
       <c r="L5">
-        <v>67.349999999999994</v>
+        <v>65.33</v>
       </c>
       <c r="M5">
-        <v>262666.2</v>
+        <v>254806.34</v>
       </c>
       <c r="N5">
-        <v>793223.71</v>
+        <v>930774.65</v>
       </c>
       <c r="O5">
-        <v>308355.53999999998</v>
+        <v>56390.67</v>
       </c>
       <c r="P5">
-        <v>0</v>
+        <v>49468.89</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -872,28 +873,28 @@
         <v>32500000</v>
       </c>
       <c r="I6">
-        <v>13023181.460000001</v>
+        <v>17566408.109999999</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>17135765.079999998</v>
+        <v>21958010.140000001</v>
       </c>
       <c r="L6">
-        <v>52.73</v>
+        <v>67.56</v>
       </c>
       <c r="M6">
-        <v>685430.6</v>
+        <v>878320.41</v>
       </c>
       <c r="N6">
-        <v>3246136.42</v>
+        <v>2986718.38</v>
       </c>
       <c r="O6">
-        <v>319876.71999999997</v>
+        <v>349100.54</v>
       </c>
       <c r="P6">
-        <v>396666.79</v>
+        <v>1183017.07</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -925,28 +926,28 @@
         <v>113750000</v>
       </c>
       <c r="I7">
-        <v>24724519.300000001</v>
+        <v>29241469.460000001</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>32532262.239999998</v>
+        <v>36551836.829999998</v>
       </c>
       <c r="L7">
-        <v>28.6</v>
+        <v>32.130000000000003</v>
       </c>
       <c r="M7">
-        <v>1301290.49</v>
+        <v>1462073.47</v>
       </c>
       <c r="N7">
-        <v>14837580.119999999</v>
+        <v>16901706.109999999</v>
       </c>
       <c r="O7">
-        <v>489653.62</v>
+        <v>473198.97</v>
       </c>
       <c r="P7">
-        <v>297833.75</v>
+        <v>1994036.11</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -978,28 +979,28 @@
         <v>39000000</v>
       </c>
       <c r="I8">
-        <v>27721316.34</v>
+        <v>33712602.560000002</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>36475416.229999997</v>
+        <v>42140753.200000003</v>
       </c>
       <c r="L8">
-        <v>93.53</v>
+        <v>108.05</v>
       </c>
       <c r="M8">
-        <v>1459016.65</v>
+        <v>1685630.13</v>
       </c>
       <c r="N8">
-        <v>1879780.61</v>
+        <v>1057479.49</v>
       </c>
       <c r="O8">
-        <v>2644626.5099999998</v>
+        <v>1554619.83</v>
       </c>
       <c r="P8">
-        <v>568183.43000000005</v>
+        <v>1910602.8</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1077,7 +1078,7 @@
         <v>40</v>
       </c>
       <c r="H2">
-        <v>1.8</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1103,7 +1104,7 @@
         <v>40</v>
       </c>
       <c r="H3">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1129,7 +1130,7 @@
         <v>40</v>
       </c>
       <c r="H4">
-        <v>1.2</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1155,7 +1156,7 @@
         <v>40</v>
       </c>
       <c r="H5">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -1207,7 +1208,7 @@
         <v>40</v>
       </c>
       <c r="H7">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -1233,7 +1234,7 @@
         <v>40</v>
       </c>
       <c r="H8">
-        <v>10.4</v>
+        <v>8.8000000000000007</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -1285,7 +1286,7 @@
         <v>42</v>
       </c>
       <c r="H10">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: cierre dia 2026-09-24_1516 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E3468A4E-9AB3-4419-BB58-3881DCD8280B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0BC11E82-0DC6-4B21-A78E-E6A15B55F29D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -667,22 +667,22 @@
         <v>0</v>
       </c>
       <c r="K2">
-        <v>3516885.56</v>
+        <v>3349414.82</v>
       </c>
       <c r="L2">
-        <v>40.520000000000003</v>
+        <v>38.590000000000003</v>
       </c>
       <c r="M2">
-        <v>140675.42000000001</v>
+        <v>133976.59</v>
       </c>
       <c r="N2">
-        <v>1173298.31</v>
+        <v>1466622.89</v>
       </c>
       <c r="O2">
-        <v>501954.16</v>
+        <v>0</v>
       </c>
       <c r="P2">
-        <v>32339.59</v>
+        <v>-25420.1</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -714,28 +714,28 @@
         <v>61320000</v>
       </c>
       <c r="I3">
-        <v>60274602.219999999</v>
+        <v>61241781.640000001</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>75343252.769999996</v>
+        <v>72906882.900000006</v>
       </c>
       <c r="L3">
-        <v>122.87</v>
+        <v>118.9</v>
       </c>
       <c r="M3">
-        <v>3013730.11</v>
+        <v>2916275.32</v>
       </c>
       <c r="N3">
-        <v>209079.56</v>
+        <v>19554.59</v>
       </c>
       <c r="O3">
-        <v>14104664.09</v>
+        <v>565637.09</v>
       </c>
       <c r="P3">
-        <v>153860.60999999999</v>
+        <v>326830.42</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -767,28 +767,28 @@
         <v>130000000</v>
       </c>
       <c r="I4">
-        <v>127386291.16</v>
+        <v>131663543.68000001</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>159232863.94999999</v>
+        <v>156742313.91</v>
       </c>
       <c r="L4">
-        <v>122.49</v>
+        <v>120.57</v>
       </c>
       <c r="M4">
-        <v>6369314.5599999996</v>
+        <v>6269692.5599999996</v>
       </c>
       <c r="N4">
-        <v>522741.77</v>
+        <v>-415885.92</v>
       </c>
       <c r="O4">
-        <v>1017675.24</v>
+        <v>381058.52</v>
       </c>
       <c r="P4">
-        <v>27847207.91</v>
+        <v>2343794.06</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -820,28 +820,28 @@
         <v>9750000</v>
       </c>
       <c r="I5">
-        <v>5096126.7300000004</v>
+        <v>5429541.6799999997</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>6370158.4100000001</v>
+        <v>6463740.0899999999</v>
       </c>
       <c r="L5">
-        <v>65.33</v>
+        <v>66.290000000000006</v>
       </c>
       <c r="M5">
-        <v>254806.34</v>
+        <v>258549.6</v>
       </c>
       <c r="N5">
-        <v>930774.65</v>
+        <v>1080114.58</v>
       </c>
       <c r="O5">
-        <v>56390.67</v>
+        <v>0</v>
       </c>
       <c r="P5">
-        <v>49468.89</v>
+        <v>1776305.96</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -873,28 +873,28 @@
         <v>32500000</v>
       </c>
       <c r="I6">
-        <v>17566408.109999999</v>
+        <v>17715847.77</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>21958010.140000001</v>
+        <v>21090294.960000001</v>
       </c>
       <c r="L6">
-        <v>67.56</v>
+        <v>64.89</v>
       </c>
       <c r="M6">
-        <v>878320.41</v>
+        <v>843611.8</v>
       </c>
       <c r="N6">
-        <v>2986718.38</v>
+        <v>3696038.06</v>
       </c>
       <c r="O6">
-        <v>349100.54</v>
+        <v>173028.51</v>
       </c>
       <c r="P6">
-        <v>1183017.07</v>
+        <v>2100481.14</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -926,28 +926,28 @@
         <v>113750000</v>
       </c>
       <c r="I7">
-        <v>29241469.460000001</v>
+        <v>31220602.260000002</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>36551836.829999998</v>
+        <v>37167383.640000001</v>
       </c>
       <c r="L7">
-        <v>32.130000000000003</v>
+        <v>32.67</v>
       </c>
       <c r="M7">
-        <v>1462073.47</v>
+        <v>1486695.35</v>
       </c>
       <c r="N7">
-        <v>16901706.109999999</v>
+        <v>20632349.440000001</v>
       </c>
       <c r="O7">
-        <v>473198.97</v>
+        <v>758561.49</v>
       </c>
       <c r="P7">
-        <v>1994036.11</v>
+        <v>641164.41</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -979,28 +979,28 @@
         <v>39000000</v>
       </c>
       <c r="I8">
-        <v>33712602.560000002</v>
+        <v>34010627.810000002</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>42140753.200000003</v>
+        <v>40488842.630000003</v>
       </c>
       <c r="L8">
-        <v>108.05</v>
+        <v>103.82</v>
       </c>
       <c r="M8">
-        <v>1685630.13</v>
+        <v>1619553.71</v>
       </c>
       <c r="N8">
-        <v>1057479.49</v>
+        <v>1247343.05</v>
       </c>
       <c r="O8">
-        <v>1554619.83</v>
+        <v>192509.06</v>
       </c>
       <c r="P8">
-        <v>1910602.8</v>
+        <v>3571862.36</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1234,7 +1234,7 @@
         <v>40</v>
       </c>
       <c r="H8">
-        <v>8.8000000000000007</v>
+        <v>8.1999999999999993</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
data: cierre dia 2026-09-25_1740 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0BC11E82-0DC6-4B21-A78E-E6A15B55F29D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{94EA6940-2BB6-41C7-BCAC-BA6061018337}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -661,28 +661,28 @@
         <v>8680000</v>
       </c>
       <c r="I2">
-        <v>2813508.45</v>
+        <v>2899704.23</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>3349414.82</v>
+        <v>3295118.44</v>
       </c>
       <c r="L2">
-        <v>38.590000000000003</v>
+        <v>37.96</v>
       </c>
       <c r="M2">
-        <v>133976.59</v>
+        <v>131804.74</v>
       </c>
       <c r="N2">
-        <v>1466622.89</v>
+        <v>1926765.26</v>
       </c>
       <c r="O2">
-        <v>0</v>
+        <v>55925.53</v>
       </c>
       <c r="P2">
-        <v>-25420.1</v>
+        <v>0</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -714,28 +714,28 @@
         <v>61320000</v>
       </c>
       <c r="I3">
-        <v>61241781.640000001</v>
+        <v>64666625.490000002</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>72906882.900000006</v>
+        <v>73484801.689999998</v>
       </c>
       <c r="L3">
-        <v>118.9</v>
+        <v>119.84</v>
       </c>
       <c r="M3">
-        <v>2916275.32</v>
+        <v>2939392.07</v>
       </c>
       <c r="N3">
-        <v>19554.59</v>
+        <v>-1115541.83</v>
       </c>
       <c r="O3">
-        <v>565637.09</v>
+        <v>4753855.7699999996</v>
       </c>
       <c r="P3">
-        <v>326830.42</v>
+        <v>122098.18</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -767,28 +767,28 @@
         <v>130000000</v>
       </c>
       <c r="I4">
-        <v>131663543.68000001</v>
+        <v>138357434.02000001</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>156742313.91</v>
+        <v>157224356.84</v>
       </c>
       <c r="L4">
-        <v>120.57</v>
+        <v>120.94</v>
       </c>
       <c r="M4">
-        <v>6269692.5599999996</v>
+        <v>6288974.2699999996</v>
       </c>
       <c r="N4">
-        <v>-415885.92</v>
+        <v>-2785811.34</v>
       </c>
       <c r="O4">
-        <v>381058.52</v>
+        <v>0</v>
       </c>
       <c r="P4">
-        <v>2343794.06</v>
+        <v>21346389.219999999</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -820,28 +820,28 @@
         <v>9750000</v>
       </c>
       <c r="I5">
-        <v>5429541.6799999997</v>
+        <v>5096126.7300000004</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>6463740.0899999999</v>
+        <v>5791053.0999999996</v>
       </c>
       <c r="L5">
-        <v>66.290000000000006</v>
+        <v>59.4</v>
       </c>
       <c r="M5">
-        <v>258549.6</v>
+        <v>231642.12</v>
       </c>
       <c r="N5">
-        <v>1080114.58</v>
+        <v>1551291.09</v>
       </c>
       <c r="O5">
         <v>0</v>
       </c>
       <c r="P5">
-        <v>1776305.96</v>
+        <v>0</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -873,28 +873,28 @@
         <v>32500000</v>
       </c>
       <c r="I6">
-        <v>17715847.77</v>
+        <v>18480791.969999999</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>21090294.960000001</v>
+        <v>21000899.960000001</v>
       </c>
       <c r="L6">
-        <v>64.89</v>
+        <v>64.62</v>
       </c>
       <c r="M6">
-        <v>843611.8</v>
+        <v>840036</v>
       </c>
       <c r="N6">
-        <v>3696038.06</v>
+        <v>4673069.34</v>
       </c>
       <c r="O6">
-        <v>173028.51</v>
+        <v>0</v>
       </c>
       <c r="P6">
-        <v>2100481.14</v>
+        <v>0</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -926,28 +926,28 @@
         <v>113750000</v>
       </c>
       <c r="I7">
-        <v>31220602.260000002</v>
+        <v>42910821.25</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>37167383.640000001</v>
+        <v>48762296.869999997</v>
       </c>
       <c r="L7">
-        <v>32.67</v>
+        <v>42.87</v>
       </c>
       <c r="M7">
-        <v>1486695.35</v>
+        <v>1950491.87</v>
       </c>
       <c r="N7">
-        <v>20632349.440000001</v>
+        <v>23613059.579999998</v>
       </c>
       <c r="O7">
-        <v>758561.49</v>
+        <v>4928307.16</v>
       </c>
       <c r="P7">
-        <v>641164.41</v>
+        <v>153654.56</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -979,28 +979,28 @@
         <v>39000000</v>
       </c>
       <c r="I8">
-        <v>34010627.810000002</v>
+        <v>35635992.009999998</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>40488842.630000003</v>
+        <v>40495445.460000001</v>
       </c>
       <c r="L8">
-        <v>103.82</v>
+        <v>103.83</v>
       </c>
       <c r="M8">
-        <v>1619553.71</v>
+        <v>1619817.82</v>
       </c>
       <c r="N8">
-        <v>1247343.05</v>
+        <v>1121336</v>
       </c>
       <c r="O8">
-        <v>192509.06</v>
+        <v>-29537.52</v>
       </c>
       <c r="P8">
-        <v>3571862.36</v>
+        <v>0</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1078,7 +1078,7 @@
         <v>40</v>
       </c>
       <c r="H2">
-        <v>1.5</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1104,7 +1104,7 @@
         <v>40</v>
       </c>
       <c r="H3">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1130,7 +1130,7 @@
         <v>40</v>
       </c>
       <c r="H4">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1182,7 +1182,7 @@
         <v>40</v>
       </c>
       <c r="H6">
-        <v>2.1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -1234,7 +1234,7 @@
         <v>40</v>
       </c>
       <c r="H8">
-        <v>8.1999999999999993</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -1260,7 +1260,7 @@
         <v>42</v>
       </c>
       <c r="H9">
-        <v>1.3</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
data: cierre dia 2026-09-28_1245 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{94EA6940-2BB6-41C7-BCAC-BA6061018337}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E7500723-F196-4781-8353-16D45829EBF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -661,25 +661,25 @@
         <v>8680000</v>
       </c>
       <c r="I2">
-        <v>2899704.23</v>
+        <v>2930398.49</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>3295118.44</v>
+        <v>3185215.76</v>
       </c>
       <c r="L2">
-        <v>37.96</v>
+        <v>36.700000000000003</v>
       </c>
       <c r="M2">
-        <v>131804.74</v>
+        <v>127408.63</v>
       </c>
       <c r="N2">
-        <v>1926765.26</v>
+        <v>2874800.75</v>
       </c>
       <c r="O2">
-        <v>55925.53</v>
+        <v>0</v>
       </c>
       <c r="P2">
         <v>0</v>
@@ -720,22 +720,22 @@
         <v>0</v>
       </c>
       <c r="K3">
-        <v>73484801.689999998</v>
+        <v>70289810.310000002</v>
       </c>
       <c r="L3">
-        <v>119.84</v>
+        <v>114.63</v>
       </c>
       <c r="M3">
-        <v>2939392.07</v>
+        <v>2811592.41</v>
       </c>
       <c r="N3">
-        <v>-1115541.83</v>
+        <v>-1673312.74</v>
       </c>
       <c r="O3">
-        <v>4753855.7699999996</v>
+        <v>7211970.4800000004</v>
       </c>
       <c r="P3">
-        <v>122098.18</v>
+        <v>1670173.09</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -767,28 +767,28 @@
         <v>130000000</v>
       </c>
       <c r="I4">
-        <v>138357434.02000001</v>
+        <v>138454036.44</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>157224356.84</v>
+        <v>150493517.87</v>
       </c>
       <c r="L4">
-        <v>120.94</v>
+        <v>115.76</v>
       </c>
       <c r="M4">
-        <v>6288974.2699999996</v>
+        <v>6019740.71</v>
       </c>
       <c r="N4">
-        <v>-2785811.34</v>
+        <v>-4227018.22</v>
       </c>
       <c r="O4">
-        <v>0</v>
+        <v>2269511.59</v>
       </c>
       <c r="P4">
-        <v>21346389.219999999</v>
+        <v>97710.18</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -826,16 +826,16 @@
         <v>0</v>
       </c>
       <c r="K5">
-        <v>5791053.0999999996</v>
+        <v>5539268.1900000004</v>
       </c>
       <c r="L5">
-        <v>59.4</v>
+        <v>56.81</v>
       </c>
       <c r="M5">
-        <v>231642.12</v>
+        <v>221570.73</v>
       </c>
       <c r="N5">
-        <v>1551291.09</v>
+        <v>2326936.63</v>
       </c>
       <c r="O5">
         <v>0</v>
@@ -879,22 +879,22 @@
         <v>0</v>
       </c>
       <c r="K6">
-        <v>21000899.960000001</v>
+        <v>20087817.350000001</v>
       </c>
       <c r="L6">
-        <v>64.62</v>
+        <v>61.81</v>
       </c>
       <c r="M6">
-        <v>840036</v>
+        <v>803512.69</v>
       </c>
       <c r="N6">
-        <v>4673069.34</v>
+        <v>7009604.0199999996</v>
       </c>
       <c r="O6">
-        <v>0</v>
+        <v>18048.23</v>
       </c>
       <c r="P6">
-        <v>0</v>
+        <v>331401.26</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -926,28 +926,28 @@
         <v>113750000</v>
       </c>
       <c r="I7">
-        <v>42910821.25</v>
+        <v>43632055.479999997</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>48762296.869999997</v>
+        <v>47426147.259999998</v>
       </c>
       <c r="L7">
-        <v>42.87</v>
+        <v>41.69</v>
       </c>
       <c r="M7">
-        <v>1950491.87</v>
+        <v>1897045.89</v>
       </c>
       <c r="N7">
-        <v>23613059.579999998</v>
+        <v>35058972.259999998</v>
       </c>
       <c r="O7">
-        <v>4928307.16</v>
+        <v>693003.37</v>
       </c>
       <c r="P7">
-        <v>153654.56</v>
+        <v>3390840.82</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -979,28 +979,28 @@
         <v>39000000</v>
       </c>
       <c r="I8">
-        <v>35635992.009999998</v>
+        <v>35977351.759999998</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>40495445.460000001</v>
+        <v>39105817.130000003</v>
       </c>
       <c r="L8">
-        <v>103.83</v>
+        <v>100.27</v>
       </c>
       <c r="M8">
-        <v>1619817.82</v>
+        <v>1564232.69</v>
       </c>
       <c r="N8">
-        <v>1121336</v>
+        <v>1511324.12</v>
       </c>
       <c r="O8">
-        <v>-29537.52</v>
+        <v>171121.52</v>
       </c>
       <c r="P8">
-        <v>0</v>
+        <v>165406.84</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1130,7 +1130,7 @@
         <v>40</v>
       </c>
       <c r="H4">
-        <v>1.3</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1234,7 +1234,7 @@
         <v>40</v>
       </c>
       <c r="H8">
-        <v>6</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
data: cierre dia 2026-09-29_1725 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E7500723-F196-4781-8353-16D45829EBF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{FC995615-4AD1-42BF-B4C9-6386A7D6C844}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -661,22 +661,22 @@
         <v>8680000</v>
       </c>
       <c r="I2">
-        <v>2930398.49</v>
+        <v>7998975.3499999996</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>3185215.76</v>
+        <v>8332265.9900000002</v>
       </c>
       <c r="L2">
-        <v>36.700000000000003</v>
+        <v>95.99</v>
       </c>
       <c r="M2">
-        <v>127408.63</v>
+        <v>333290.64</v>
       </c>
       <c r="N2">
-        <v>2874800.75</v>
+        <v>681024.65</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -714,28 +714,28 @@
         <v>61320000</v>
       </c>
       <c r="I3">
-        <v>64666625.490000002</v>
+        <v>69983715.930000007</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>70289810.310000002</v>
+        <v>72899704.090000004</v>
       </c>
       <c r="L3">
-        <v>114.63</v>
+        <v>118.88</v>
       </c>
       <c r="M3">
-        <v>2811592.41</v>
+        <v>2915988.16</v>
       </c>
       <c r="N3">
-        <v>-1673312.74</v>
+        <v>-8663715.9299999997</v>
       </c>
       <c r="O3">
-        <v>7211970.4800000004</v>
+        <v>7018214.7599999998</v>
       </c>
       <c r="P3">
-        <v>1670173.09</v>
+        <v>481783.87</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -767,28 +767,28 @@
         <v>130000000</v>
       </c>
       <c r="I4">
-        <v>138454036.44</v>
+        <v>146397924.81</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>150493517.87</v>
+        <v>152497838.34</v>
       </c>
       <c r="L4">
-        <v>115.76</v>
+        <v>117.31</v>
       </c>
       <c r="M4">
-        <v>6019740.71</v>
+        <v>6099913.5300000003</v>
       </c>
       <c r="N4">
-        <v>-4227018.22</v>
+        <v>-16397924.810000001</v>
       </c>
       <c r="O4">
-        <v>2269511.59</v>
+        <v>15737357.01</v>
       </c>
       <c r="P4">
-        <v>97710.18</v>
+        <v>2250370.58</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -820,28 +820,28 @@
         <v>9750000</v>
       </c>
       <c r="I5">
-        <v>5096126.7300000004</v>
+        <v>6710789.6699999999</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>5539268.1900000004</v>
+        <v>6990405.9100000001</v>
       </c>
       <c r="L5">
-        <v>56.81</v>
+        <v>71.7</v>
       </c>
       <c r="M5">
-        <v>221570.73</v>
+        <v>279616.24</v>
       </c>
       <c r="N5">
-        <v>2326936.63</v>
+        <v>3039210.33</v>
       </c>
       <c r="O5">
-        <v>0</v>
+        <v>105469</v>
       </c>
       <c r="P5">
-        <v>0</v>
+        <v>308355.53999999998</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -873,28 +873,28 @@
         <v>32500000</v>
       </c>
       <c r="I6">
-        <v>18480791.969999999</v>
+        <v>19082752.07</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>20087817.350000001</v>
+        <v>19877866.739999998</v>
       </c>
       <c r="L6">
-        <v>61.81</v>
+        <v>61.16</v>
       </c>
       <c r="M6">
-        <v>803512.69</v>
+        <v>795114.67</v>
       </c>
       <c r="N6">
-        <v>7009604.0199999996</v>
+        <v>13417247.93</v>
       </c>
       <c r="O6">
-        <v>18048.23</v>
+        <v>4543226.6500000004</v>
       </c>
       <c r="P6">
-        <v>331401.26</v>
+        <v>319876.71999999997</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -926,28 +926,28 @@
         <v>113750000</v>
       </c>
       <c r="I7">
-        <v>43632055.479999997</v>
+        <v>60708631.68</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>47426147.259999998</v>
+        <v>63238158</v>
       </c>
       <c r="L7">
-        <v>41.69</v>
+        <v>55.59</v>
       </c>
       <c r="M7">
-        <v>1897045.89</v>
+        <v>2529526.3199999998</v>
       </c>
       <c r="N7">
-        <v>35058972.259999998</v>
+        <v>53041368.32</v>
       </c>
       <c r="O7">
-        <v>693003.37</v>
+        <v>4516950.16</v>
       </c>
       <c r="P7">
-        <v>3390840.82</v>
+        <v>489653.62</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -979,28 +979,28 @@
         <v>39000000</v>
       </c>
       <c r="I8">
-        <v>35977351.759999998</v>
+        <v>38501758.899999999</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>39105817.130000003</v>
+        <v>40105998.859999999</v>
       </c>
       <c r="L8">
-        <v>100.27</v>
+        <v>102.84</v>
       </c>
       <c r="M8">
-        <v>1564232.69</v>
+        <v>1604239.95</v>
       </c>
       <c r="N8">
-        <v>1511324.12</v>
+        <v>498241.1</v>
       </c>
       <c r="O8">
-        <v>171121.52</v>
+        <v>5991286.2300000004</v>
       </c>
       <c r="P8">
-        <v>165406.84</v>
+        <v>2644626.5099999998</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1182,7 +1182,7 @@
         <v>40</v>
       </c>
       <c r="H6">
-        <v>2</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -1234,7 +1234,7 @@
         <v>40</v>
       </c>
       <c r="H8">
-        <v>5.9</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -1260,7 +1260,7 @@
         <v>42</v>
       </c>
       <c r="H9">
-        <v>1.2</v>
+        <v>1.1000000000000001</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -1286,7 +1286,7 @@
         <v>42</v>
       </c>
       <c r="H10">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: cierre dia 2026-09-30_1552 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FC995615-4AD1-42BF-B4C9-6386A7D6C844}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{186C3BB4-C00A-4528-B602-DAE5F58F97B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -661,28 +661,28 @@
         <v>8680000</v>
       </c>
       <c r="I2">
-        <v>7998975.3499999996</v>
+        <v>8371471.5700000003</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>8332265.9900000002</v>
+        <v>8371471.5700000003</v>
       </c>
       <c r="L2">
-        <v>95.99</v>
+        <v>96.45</v>
       </c>
       <c r="M2">
-        <v>333290.64</v>
+        <v>334858.86</v>
       </c>
       <c r="N2">
-        <v>681024.65</v>
+        <v>0</v>
       </c>
       <c r="O2">
-        <v>0</v>
+        <v>86195.78</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>501954.16</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -714,28 +714,28 @@
         <v>61320000</v>
       </c>
       <c r="I3">
-        <v>69983715.930000007</v>
+        <v>70280526.400000006</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>72899704.090000004</v>
+        <v>70280526.400000006</v>
       </c>
       <c r="L3">
-        <v>118.88</v>
+        <v>114.61</v>
       </c>
       <c r="M3">
-        <v>2915988.16</v>
+        <v>2811221.06</v>
       </c>
       <c r="N3">
-        <v>-8663715.9299999997</v>
+        <v>0</v>
       </c>
       <c r="O3">
-        <v>7018214.7599999998</v>
+        <v>1205219.8</v>
       </c>
       <c r="P3">
-        <v>481783.87</v>
+        <v>14104664.09</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -767,28 +767,28 @@
         <v>130000000</v>
       </c>
       <c r="I4">
-        <v>146397924.81</v>
+        <v>148576900.31999999</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>152497838.34</v>
+        <v>148576900.31999999</v>
       </c>
       <c r="L4">
-        <v>117.31</v>
+        <v>114.29</v>
       </c>
       <c r="M4">
-        <v>6099913.5300000003</v>
+        <v>5943076.0099999998</v>
       </c>
       <c r="N4">
-        <v>-16397924.810000001</v>
+        <v>0</v>
       </c>
       <c r="O4">
-        <v>15737357.01</v>
+        <v>4227899.84</v>
       </c>
       <c r="P4">
-        <v>2250370.58</v>
+        <v>1017675.24</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -820,28 +820,28 @@
         <v>9750000</v>
       </c>
       <c r="I5">
-        <v>6710789.6699999999</v>
+        <v>7780540.3300000001</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>6990405.9100000001</v>
+        <v>7780540.3300000001</v>
       </c>
       <c r="L5">
-        <v>71.7</v>
+        <v>79.8</v>
       </c>
       <c r="M5">
-        <v>279616.24</v>
+        <v>311221.61</v>
       </c>
       <c r="N5">
-        <v>3039210.33</v>
+        <v>0</v>
       </c>
       <c r="O5">
-        <v>105469</v>
+        <v>0</v>
       </c>
       <c r="P5">
-        <v>308355.53999999998</v>
+        <v>56390.67</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -873,28 +873,28 @@
         <v>32500000</v>
       </c>
       <c r="I6">
-        <v>19082752.07</v>
+        <v>19972946.93</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>19877866.739999998</v>
+        <v>19972946.93</v>
       </c>
       <c r="L6">
-        <v>61.16</v>
+        <v>61.46</v>
       </c>
       <c r="M6">
-        <v>795114.67</v>
+        <v>798917.88</v>
       </c>
       <c r="N6">
-        <v>13417247.93</v>
+        <v>0</v>
       </c>
       <c r="O6">
-        <v>4543226.6500000004</v>
+        <v>149439.66</v>
       </c>
       <c r="P6">
-        <v>319876.71999999997</v>
+        <v>349100.54</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -932,22 +932,22 @@
         <v>0</v>
       </c>
       <c r="K7">
-        <v>63238158</v>
+        <v>60708631.68</v>
       </c>
       <c r="L7">
-        <v>55.59</v>
+        <v>53.37</v>
       </c>
       <c r="M7">
-        <v>2529526.3199999998</v>
+        <v>2428345.27</v>
       </c>
       <c r="N7">
-        <v>53041368.32</v>
+        <v>0</v>
       </c>
       <c r="O7">
-        <v>4516950.16</v>
+        <v>2028360.96</v>
       </c>
       <c r="P7">
-        <v>489653.62</v>
+        <v>473198.97</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -979,28 +979,28 @@
         <v>39000000</v>
       </c>
       <c r="I8">
-        <v>38501758.899999999</v>
+        <v>38496559.009999998</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>40105998.859999999</v>
+        <v>38496559.009999998</v>
       </c>
       <c r="L8">
-        <v>102.84</v>
+        <v>98.71</v>
       </c>
       <c r="M8">
-        <v>1604239.95</v>
+        <v>1539862.36</v>
       </c>
       <c r="N8">
-        <v>498241.1</v>
+        <v>0</v>
       </c>
       <c r="O8">
-        <v>5991286.2300000004</v>
+        <v>298025.24</v>
       </c>
       <c r="P8">
-        <v>2644626.5099999998</v>
+        <v>1554619.83</v>
       </c>
       <c r="Q8">
         <v>0</v>
@@ -1078,7 +1078,7 @@
         <v>40</v>
       </c>
       <c r="H2">
-        <v>1.4</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1104,7 +1104,7 @@
         <v>40</v>
       </c>
       <c r="H3">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
data: cierre dia 2026-10-02_1528 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{021F16E8-130E-4F0A-8D2E-C3E66D52D9DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A97DD129-7AC8-460A-907A-C23F915A4E14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -660,28 +660,28 @@
         <v>8680000</v>
       </c>
       <c r="I2">
-        <v>230363.61</v>
+        <v>216245.74</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>5989453.8799999999</v>
+        <v>2811194.65</v>
       </c>
       <c r="L2">
-        <v>69</v>
+        <v>32.39</v>
       </c>
       <c r="M2">
-        <v>230363.61</v>
+        <v>108122.87</v>
       </c>
       <c r="N2">
-        <v>337985.46</v>
+        <v>352656.43</v>
       </c>
       <c r="O2">
-        <v>0</v>
+        <v>30694.26</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>55925.53</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -713,28 +713,28 @@
         <v>61320000</v>
       </c>
       <c r="I3">
-        <v>685624.04</v>
+        <v>1236890.27</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>17826224.989999998</v>
+        <v>16079573.449999999</v>
       </c>
       <c r="L3">
-        <v>29.07</v>
+        <v>26.22</v>
       </c>
       <c r="M3">
-        <v>685624.04</v>
+        <v>618445.13</v>
       </c>
       <c r="N3">
-        <v>2425375.04</v>
+        <v>2503462.91</v>
       </c>
       <c r="O3">
-        <v>3186803.47</v>
+        <v>0</v>
       </c>
       <c r="P3">
-        <v>565637.09</v>
+        <v>4753855.7699999996</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -766,28 +766,28 @@
         <v>130000000</v>
       </c>
       <c r="I4">
-        <v>2003098.56</v>
+        <v>2804917.28</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>52080562.490000002</v>
+        <v>36463924.619999997</v>
       </c>
       <c r="L4">
-        <v>40.06</v>
+        <v>28.05</v>
       </c>
       <c r="M4">
-        <v>2003098.56</v>
+        <v>1402458.64</v>
       </c>
       <c r="N4">
-        <v>5119876.0599999996</v>
+        <v>5299795.1100000003</v>
       </c>
       <c r="O4">
-        <v>6743243.0099999998</v>
+        <v>96602.42</v>
       </c>
       <c r="P4">
-        <v>381058.52</v>
+        <v>0</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -819,22 +819,22 @@
         <v>9750000</v>
       </c>
       <c r="I5">
-        <v>404459.3</v>
+        <v>449062.15</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>10515941.77</v>
+        <v>5837807.96</v>
       </c>
       <c r="L5">
-        <v>107.86</v>
+        <v>59.87</v>
       </c>
       <c r="M5">
-        <v>404459.3</v>
+        <v>224531.08</v>
       </c>
       <c r="N5">
-        <v>373821.63</v>
+        <v>387539.08</v>
       </c>
       <c r="O5">
         <v>0</v>
@@ -872,28 +872,28 @@
         <v>32500000</v>
       </c>
       <c r="I6">
-        <v>735735.34</v>
+        <v>1173005.22</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>19129118.850000001</v>
+        <v>15249067.91</v>
       </c>
       <c r="L6">
-        <v>58.86</v>
+        <v>46.92</v>
       </c>
       <c r="M6">
-        <v>735735.34</v>
+        <v>586502.61</v>
       </c>
       <c r="N6">
-        <v>1270570.5900000001</v>
+        <v>1305291.45</v>
       </c>
       <c r="O6">
-        <v>764944.2</v>
+        <v>0</v>
       </c>
       <c r="P6">
-        <v>173028.51</v>
+        <v>0</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -925,28 +925,28 @@
         <v>113750000</v>
       </c>
       <c r="I7">
-        <v>2122541.31</v>
+        <v>2590148.4500000002</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>55186074.109999999</v>
+        <v>33671929.880000003</v>
       </c>
       <c r="L7">
-        <v>48.52</v>
+        <v>29.6</v>
       </c>
       <c r="M7">
-        <v>2122541.31</v>
+        <v>1295074.23</v>
       </c>
       <c r="N7">
-        <v>4465098.3499999996</v>
+        <v>4631660.4800000004</v>
       </c>
       <c r="O7">
-        <v>11640990.82</v>
+        <v>721234.23</v>
       </c>
       <c r="P7">
-        <v>758561.49</v>
+        <v>4928307.16</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -978,28 +978,28 @@
         <v>39000000</v>
       </c>
       <c r="I8">
-        <v>2154787.64</v>
+        <v>3180470.81</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>56024478.670000002</v>
+        <v>41346120.560000002</v>
       </c>
       <c r="L8">
-        <v>143.65</v>
+        <v>106.02</v>
       </c>
       <c r="M8">
-        <v>2154787.64</v>
+        <v>1590235.41</v>
       </c>
       <c r="N8">
-        <v>1473808.49</v>
+        <v>1492480.38</v>
       </c>
       <c r="O8">
-        <v>2144511.04</v>
+        <v>0</v>
       </c>
       <c r="P8">
-        <v>192509.06</v>
+        <v>-29537.52</v>
       </c>
       <c r="Q8">
         <v>0</v>

</xml_diff>

<commit_message>
data: cierre dia 2026-10-04_1814 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A97DD129-7AC8-460A-907A-C23F915A4E14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{AA124A10-6510-496E-B191-86D5AABB53E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -660,28 +660,28 @@
         <v>8680000</v>
       </c>
       <c r="I2">
-        <v>216245.74</v>
+        <v>340310.71</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>2811194.65</v>
+        <v>2949359.47</v>
       </c>
       <c r="L2">
-        <v>32.39</v>
+        <v>33.979999999999997</v>
       </c>
       <c r="M2">
-        <v>108122.87</v>
+        <v>113436.9</v>
       </c>
       <c r="N2">
-        <v>352656.43</v>
+        <v>362595.19</v>
       </c>
       <c r="O2">
-        <v>30694.26</v>
+        <v>5068576.8600000003</v>
       </c>
       <c r="P2">
-        <v>55925.53</v>
+        <v>0</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -713,28 +713,28 @@
         <v>61320000</v>
       </c>
       <c r="I3">
-        <v>1236890.27</v>
+        <v>1268150.55</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>16079573.449999999</v>
+        <v>10990638.1</v>
       </c>
       <c r="L3">
-        <v>26.22</v>
+        <v>17.920000000000002</v>
       </c>
       <c r="M3">
-        <v>618445.13</v>
+        <v>422716.85</v>
       </c>
       <c r="N3">
-        <v>2503462.91</v>
+        <v>2610949.98</v>
       </c>
       <c r="O3">
-        <v>0</v>
+        <v>4543063.41</v>
       </c>
       <c r="P3">
-        <v>4753855.7699999996</v>
+        <v>2352908.59</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -766,28 +766,28 @@
         <v>130000000</v>
       </c>
       <c r="I4">
-        <v>2804917.28</v>
+        <v>6725069.5700000003</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>36463924.619999997</v>
+        <v>58283936.240000002</v>
       </c>
       <c r="L4">
-        <v>28.05</v>
+        <v>44.83</v>
       </c>
       <c r="M4">
-        <v>1402458.64</v>
+        <v>2241689.86</v>
       </c>
       <c r="N4">
-        <v>5299795.1100000003</v>
+        <v>5359779.58</v>
       </c>
       <c r="O4">
-        <v>96602.42</v>
+        <v>6636560.2000000002</v>
       </c>
       <c r="P4">
-        <v>0</v>
+        <v>14130294.039999999</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -825,22 +825,22 @@
         <v>0</v>
       </c>
       <c r="K5">
-        <v>5837807.96</v>
+        <v>3891871.97</v>
       </c>
       <c r="L5">
-        <v>59.87</v>
+        <v>39.92</v>
       </c>
       <c r="M5">
-        <v>224531.08</v>
+        <v>149687.38</v>
       </c>
       <c r="N5">
-        <v>387539.08</v>
+        <v>404388.6</v>
       </c>
       <c r="O5">
         <v>0</v>
       </c>
       <c r="P5">
-        <v>0</v>
+        <v>2397583.9300000002</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -872,28 +872,28 @@
         <v>32500000</v>
       </c>
       <c r="I6">
-        <v>1173005.22</v>
+        <v>1203882.73</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>15249067.91</v>
+        <v>10433650.33</v>
       </c>
       <c r="L6">
-        <v>46.92</v>
+        <v>32.1</v>
       </c>
       <c r="M6">
-        <v>586502.61</v>
+        <v>401294.24</v>
       </c>
       <c r="N6">
-        <v>1305291.45</v>
+        <v>1360700.75</v>
       </c>
       <c r="O6">
         <v>0</v>
       </c>
       <c r="P6">
-        <v>0</v>
+        <v>2551764.06</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -925,28 +925,28 @@
         <v>113750000</v>
       </c>
       <c r="I7">
-        <v>2590148.4500000002</v>
+        <v>2964226.83</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>33671929.880000003</v>
+        <v>25689965.859999999</v>
       </c>
       <c r="L7">
-        <v>29.6</v>
+        <v>22.58</v>
       </c>
       <c r="M7">
-        <v>1295074.23</v>
+        <v>988075.61</v>
       </c>
       <c r="N7">
-        <v>4631660.4800000004</v>
+        <v>4816772.75</v>
       </c>
       <c r="O7">
-        <v>721234.23</v>
+        <v>16958630.75</v>
       </c>
       <c r="P7">
-        <v>4928307.16</v>
+        <v>3086198.56</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -978,28 +978,28 @@
         <v>39000000</v>
       </c>
       <c r="I8">
-        <v>3180470.81</v>
+        <v>3242991.38</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>41346120.560000002</v>
+        <v>28105925.32</v>
       </c>
       <c r="L8">
-        <v>106.02</v>
+        <v>72.069999999999993</v>
       </c>
       <c r="M8">
-        <v>1590235.41</v>
+        <v>1080997.1299999999</v>
       </c>
       <c r="N8">
-        <v>1492480.38</v>
+        <v>1554652.55</v>
       </c>
       <c r="O8">
         <v>0</v>
       </c>
       <c r="P8">
-        <v>-29537.52</v>
+        <v>12873978.34</v>
       </c>
       <c r="Q8">
         <v>0</v>

</xml_diff>

<commit_message>
data: cierre dia 2026-10-05_1717 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AA124A10-6510-496E-B191-86D5AABB53E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{41C95202-0D22-4E70-9B5A-076687575703}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Avance" sheetId="1" r:id="rId1"/>
@@ -572,8 +572,8 @@
     <col min="4" max="4" width="16" customWidth="1"/>
     <col min="5" max="7" width="25" customWidth="1"/>
     <col min="8" max="8" width="15" customWidth="1"/>
-    <col min="9" max="9" width="12" customWidth="1"/>
-    <col min="10" max="11" width="13" customWidth="1"/>
+    <col min="9" max="10" width="13" customWidth="1"/>
+    <col min="11" max="11" width="14" customWidth="1"/>
     <col min="12" max="13" width="12" customWidth="1"/>
     <col min="14" max="14" width="16" customWidth="1"/>
     <col min="15" max="15" width="14" customWidth="1"/>
@@ -660,25 +660,25 @@
         <v>8680000</v>
       </c>
       <c r="I2">
-        <v>340310.71</v>
+        <v>401699.24</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>2949359.47</v>
+        <v>2611045.0299999998</v>
       </c>
       <c r="L2">
-        <v>33.979999999999997</v>
+        <v>30.08</v>
       </c>
       <c r="M2">
-        <v>113436.9</v>
+        <v>100424.81</v>
       </c>
       <c r="N2">
-        <v>362595.19</v>
+        <v>376286.4</v>
       </c>
       <c r="O2">
-        <v>5068576.8600000003</v>
+        <v>0</v>
       </c>
       <c r="P2">
         <v>0</v>
@@ -713,28 +713,28 @@
         <v>61320000</v>
       </c>
       <c r="I3">
-        <v>1268150.55</v>
+        <v>14903072.27</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>10990638.1</v>
+        <v>96869969.739999995</v>
       </c>
       <c r="L3">
-        <v>17.920000000000002</v>
+        <v>157.97</v>
       </c>
       <c r="M3">
-        <v>422716.85</v>
+        <v>3725768.07</v>
       </c>
       <c r="N3">
-        <v>2610949.98</v>
+        <v>2109860.35</v>
       </c>
       <c r="O3">
-        <v>4543063.41</v>
+        <v>1070837.51</v>
       </c>
       <c r="P3">
-        <v>2352908.59</v>
+        <v>7227409.2300000004</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -766,28 +766,28 @@
         <v>130000000</v>
       </c>
       <c r="I4">
-        <v>6725069.5700000003</v>
+        <v>31576974.850000001</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>58283936.240000002</v>
+        <v>205250336.50999999</v>
       </c>
       <c r="L4">
-        <v>44.83</v>
+        <v>157.88</v>
       </c>
       <c r="M4">
-        <v>2241689.86</v>
+        <v>7894243.71</v>
       </c>
       <c r="N4">
-        <v>5359779.58</v>
+        <v>4473773.87</v>
       </c>
       <c r="O4">
-        <v>6636560.2000000002</v>
+        <v>2527938.5600000001</v>
       </c>
       <c r="P4">
-        <v>14130294.039999999</v>
+        <v>2437355.81</v>
       </c>
       <c r="Q4">
         <v>0</v>
@@ -825,22 +825,22 @@
         <v>0</v>
       </c>
       <c r="K5">
-        <v>3891871.97</v>
+        <v>2918903.98</v>
       </c>
       <c r="L5">
-        <v>39.92</v>
+        <v>29.94</v>
       </c>
       <c r="M5">
-        <v>149687.38</v>
+        <v>112265.54</v>
       </c>
       <c r="N5">
-        <v>404388.6</v>
+        <v>422769.9</v>
       </c>
       <c r="O5">
-        <v>0</v>
+        <v>1614662.94</v>
       </c>
       <c r="P5">
-        <v>2397583.9300000002</v>
+        <v>0</v>
       </c>
       <c r="Q5">
         <v>0</v>
@@ -872,28 +872,28 @@
         <v>32500000</v>
       </c>
       <c r="I6">
-        <v>1203882.73</v>
+        <v>1294037.01</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>10433650.33</v>
+        <v>8411240.5700000003</v>
       </c>
       <c r="L6">
-        <v>32.1</v>
+        <v>25.88</v>
       </c>
       <c r="M6">
-        <v>401294.24</v>
+        <v>323509.25</v>
       </c>
       <c r="N6">
-        <v>1360700.75</v>
+        <v>1418452.86</v>
       </c>
       <c r="O6">
-        <v>0</v>
+        <v>617398.85</v>
       </c>
       <c r="P6">
-        <v>2551764.06</v>
+        <v>18048.23</v>
       </c>
       <c r="Q6">
         <v>0</v>
@@ -925,28 +925,28 @@
         <v>113750000</v>
       </c>
       <c r="I7">
-        <v>2964226.83</v>
+        <v>4585072.43</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>25689965.859999999</v>
+        <v>29802970.760000002</v>
       </c>
       <c r="L7">
-        <v>22.58</v>
+        <v>26.2</v>
       </c>
       <c r="M7">
-        <v>988075.61</v>
+        <v>1146268.1100000001</v>
       </c>
       <c r="N7">
-        <v>4816772.75</v>
+        <v>4962042.16</v>
       </c>
       <c r="O7">
-        <v>16958630.75</v>
+        <v>909080.77</v>
       </c>
       <c r="P7">
-        <v>3086198.56</v>
+        <v>903412.98</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -978,28 +978,28 @@
         <v>39000000</v>
       </c>
       <c r="I8">
-        <v>3242991.38</v>
+        <v>11216809.310000001</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>28105925.32</v>
+        <v>72909260.519999996</v>
       </c>
       <c r="L8">
-        <v>72.069999999999993</v>
+        <v>186.95</v>
       </c>
       <c r="M8">
-        <v>1080997.1299999999</v>
+        <v>2804202.33</v>
       </c>
       <c r="N8">
-        <v>1554652.55</v>
+        <v>1262872.3</v>
       </c>
       <c r="O8">
-        <v>0</v>
+        <v>3065018.26</v>
       </c>
       <c r="P8">
-        <v>12873978.34</v>
+        <v>171121.52</v>
       </c>
       <c r="Q8">
         <v>0</v>

</xml_diff>

<commit_message>
data: cierre dia 2026-10-06_1855 — datasets + inputs actualizados
</commit_message>
<xml_diff>
--- a/01_INPUTS/resultado.xlsx
+++ b/01_INPUTS/resultado.xlsx
@@ -3,20 +3,20 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{41C95202-0D22-4E70-9B5A-076687575703}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{EEF04987-A540-4287-BCFF-947C0618D7CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Avance" sheetId="1" r:id="rId1"/>
-    <sheet name="Rechazos" sheetId="5" r:id="rId2"/>
+    <sheet name="Rechazos" sheetId="4" r:id="rId2"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="42">
   <si>
     <t>SupervisorCodigo</t>
   </si>
@@ -43,9 +43,6 @@
   </si>
   <si>
     <t>Acumulado</t>
-  </si>
-  <si>
-    <t>AcumuladoMN</t>
   </si>
   <si>
     <t>Tendencia</t>
@@ -200,9 +197,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table0" displayName="Table0" ref="A1:Q8">
-  <autoFilter ref="A1:Q8" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
-  <tableColumns count="17">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table0" displayName="Table0" ref="A1:P8">
+  <autoFilter ref="A1:P8" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <tableColumns count="16">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="SupervisorCodigo" totalsRowLabel="Total"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="SupervisorNombre"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="VendedorId"/>
@@ -212,31 +209,30 @@
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="GrupoNombre"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="ValorObjetivo"/>
     <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Acumulado"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="AcumuladoMN"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Tendencia"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Avance"/>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Promedio"/>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="MediaNecesaria"/>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="UltimaVisita"/>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="PenultimaVisita"/>
-    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="Real"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Tendencia"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Avance"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Promedio"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="MediaNecesaria"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="UltimaVisita"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="PenultimaVisita"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Real"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium6" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="Table4" displayName="Table4" ref="A1:H10">
-  <autoFilter ref="A1:H10" xr:uid="{00000000-0009-0000-0100-000005000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="Table3" displayName="Table3" ref="A1:H10">
+  <autoFilter ref="A1:H10" xr:uid="{00000000-0009-0000-0100-000004000000}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="SupervisorId" totalsRowLabel="Total"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="SupervisorCodigo"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0400-000003000000}" name="SupervisorNombre"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0400-000004000000}" name="VendedorId"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0400-000005000000}" name="VendedorCodigo"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0400-000006000000}" name="VendedorNombre"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0400-000007000000}" name="Origen"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0400-000008000000}" name="PorcRechazo"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="SupervisorId" totalsRowLabel="Total"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="SupervisorCodigo"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="SupervisorNombre"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0300-000004000000}" name="VendedorId"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0300-000005000000}" name="VendedorCodigo"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0300-000006000000}" name="VendedorNombre"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0300-000007000000}" name="Origen"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0300-000008000000}" name="PorcRechazo"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium6" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -564,7 +560,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q8"/>
+  <dimension ref="A1:P8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="18" customWidth="1"/>
@@ -572,16 +568,16 @@
     <col min="4" max="4" width="16" customWidth="1"/>
     <col min="5" max="7" width="25" customWidth="1"/>
     <col min="8" max="8" width="15" customWidth="1"/>
-    <col min="9" max="10" width="13" customWidth="1"/>
-    <col min="11" max="11" width="14" customWidth="1"/>
-    <col min="12" max="13" width="12" customWidth="1"/>
-    <col min="14" max="14" width="16" customWidth="1"/>
-    <col min="15" max="15" width="14" customWidth="1"/>
-    <col min="16" max="16" width="17" customWidth="1"/>
-    <col min="17" max="17" width="12" customWidth="1"/>
+    <col min="9" max="9" width="13" customWidth="1"/>
+    <col min="10" max="10" width="14" customWidth="1"/>
+    <col min="11" max="12" width="12" customWidth="1"/>
+    <col min="13" max="13" width="16" customWidth="1"/>
+    <col min="14" max="14" width="14" customWidth="1"/>
+    <col min="15" max="15" width="17" customWidth="1"/>
+    <col min="16" max="16" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -630,31 +626,28 @@
       <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="B2" t="s">
         <v>17</v>
-      </c>
-      <c r="B2" t="s">
-        <v>18</v>
       </c>
       <c r="C2">
         <v>105007</v>
       </c>
       <c r="D2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E2" t="s">
         <v>19</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>20</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>21</v>
-      </c>
-      <c r="G2" t="s">
-        <v>22</v>
       </c>
       <c r="H2">
         <v>8680000</v>
@@ -663,19 +656,19 @@
         <v>401699.24</v>
       </c>
       <c r="J2">
-        <v>0</v>
+        <v>2088836.03</v>
       </c>
       <c r="K2">
-        <v>2611045.0299999998</v>
+        <v>24.06</v>
       </c>
       <c r="L2">
-        <v>30.08</v>
+        <v>80339.850000000006</v>
       </c>
       <c r="M2">
-        <v>100424.81</v>
+        <v>394204.8</v>
       </c>
       <c r="N2">
-        <v>376286.4</v>
+        <v>357149.09</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -683,325 +676,304 @@
       <c r="P2">
         <v>0</v>
       </c>
-      <c r="Q2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" t="s">
         <v>17</v>
-      </c>
-      <c r="B3" t="s">
-        <v>18</v>
       </c>
       <c r="C3">
         <v>120039</v>
       </c>
       <c r="D3" t="s">
+        <v>22</v>
+      </c>
+      <c r="E3" t="s">
         <v>23</v>
       </c>
-      <c r="E3" t="s">
-        <v>24</v>
-      </c>
       <c r="F3" t="s">
+        <v>20</v>
+      </c>
+      <c r="G3" t="s">
         <v>21</v>
-      </c>
-      <c r="G3" t="s">
-        <v>22</v>
       </c>
       <c r="H3">
         <v>61320000</v>
       </c>
       <c r="I3">
-        <v>14903072.27</v>
+        <v>17675084.59</v>
       </c>
       <c r="J3">
-        <v>0</v>
+        <v>91910439.879999995</v>
       </c>
       <c r="K3">
-        <v>96869969.739999995</v>
+        <v>149.88999999999999</v>
       </c>
       <c r="L3">
-        <v>157.97</v>
+        <v>3535016.92</v>
       </c>
       <c r="M3">
-        <v>3725768.07</v>
+        <v>2078329.31</v>
       </c>
       <c r="N3">
-        <v>2109860.35</v>
+        <v>678869.65</v>
       </c>
       <c r="O3">
-        <v>1070837.51</v>
+        <v>7018214.7599999998</v>
       </c>
       <c r="P3">
-        <v>7227409.2300000004</v>
-      </c>
-      <c r="Q3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B4" t="s">
         <v>25</v>
-      </c>
-      <c r="B4" t="s">
-        <v>26</v>
       </c>
       <c r="C4">
         <v>105008</v>
       </c>
       <c r="D4" t="s">
+        <v>26</v>
+      </c>
+      <c r="E4" t="s">
         <v>27</v>
       </c>
-      <c r="E4" t="s">
-        <v>28</v>
-      </c>
       <c r="F4" t="s">
+        <v>20</v>
+      </c>
+      <c r="G4" t="s">
         <v>21</v>
-      </c>
-      <c r="G4" t="s">
-        <v>22</v>
       </c>
       <c r="H4">
         <v>130000000</v>
       </c>
       <c r="I4">
-        <v>31576974.850000001</v>
+        <v>32802479.870000001</v>
       </c>
       <c r="J4">
-        <v>0</v>
+        <v>170572895.33000001</v>
       </c>
       <c r="K4">
-        <v>205250336.50999999</v>
+        <v>131.21</v>
       </c>
       <c r="L4">
-        <v>157.88</v>
+        <v>6560495.9699999997</v>
       </c>
       <c r="M4">
-        <v>7894243.71</v>
+        <v>4628453.34</v>
       </c>
       <c r="N4">
-        <v>4473773.87</v>
+        <v>1976419.66</v>
       </c>
       <c r="O4">
-        <v>2527938.5600000001</v>
+        <v>15869358.35</v>
       </c>
       <c r="P4">
-        <v>2437355.81</v>
-      </c>
-      <c r="Q4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>24</v>
+      </c>
+      <c r="B5" t="s">
         <v>25</v>
-      </c>
-      <c r="B5" t="s">
-        <v>26</v>
       </c>
       <c r="C5">
         <v>105003</v>
       </c>
       <c r="D5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E5" t="s">
         <v>29</v>
       </c>
-      <c r="E5" t="s">
-        <v>30</v>
-      </c>
       <c r="F5" t="s">
+        <v>20</v>
+      </c>
+      <c r="G5" t="s">
         <v>21</v>
-      </c>
-      <c r="G5" t="s">
-        <v>22</v>
       </c>
       <c r="H5">
         <v>9750000</v>
       </c>
       <c r="I5">
-        <v>449062.15</v>
+        <v>463795.4</v>
       </c>
       <c r="J5">
-        <v>0</v>
+        <v>2411736.06</v>
       </c>
       <c r="K5">
-        <v>2918903.98</v>
+        <v>24.74</v>
       </c>
       <c r="L5">
-        <v>29.94</v>
+        <v>92759.08</v>
       </c>
       <c r="M5">
-        <v>112265.54</v>
+        <v>442200.22</v>
       </c>
       <c r="N5">
-        <v>422769.9</v>
+        <v>1069750.6599999999</v>
       </c>
       <c r="O5">
-        <v>1614662.94</v>
+        <v>105469</v>
       </c>
       <c r="P5">
         <v>0</v>
       </c>
-      <c r="Q5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>24</v>
+      </c>
+      <c r="B6" t="s">
         <v>25</v>
-      </c>
-      <c r="B6" t="s">
-        <v>26</v>
       </c>
       <c r="C6">
         <v>105004</v>
       </c>
       <c r="D6" t="s">
+        <v>30</v>
+      </c>
+      <c r="E6" t="s">
         <v>31</v>
       </c>
-      <c r="E6" t="s">
-        <v>32</v>
-      </c>
       <c r="F6" t="s">
+        <v>20</v>
+      </c>
+      <c r="G6" t="s">
         <v>21</v>
-      </c>
-      <c r="G6" t="s">
-        <v>22</v>
       </c>
       <c r="H6">
         <v>32500000</v>
       </c>
       <c r="I6">
-        <v>1294037.01</v>
+        <v>2014498.63</v>
       </c>
       <c r="J6">
-        <v>0</v>
+        <v>10475392.85</v>
       </c>
       <c r="K6">
-        <v>8411240.5700000003</v>
+        <v>32.229999999999997</v>
       </c>
       <c r="L6">
-        <v>25.88</v>
+        <v>402899.73</v>
       </c>
       <c r="M6">
-        <v>323509.25</v>
+        <v>1451690.54</v>
       </c>
       <c r="N6">
-        <v>1418452.86</v>
+        <v>1487554.24</v>
       </c>
       <c r="O6">
-        <v>617398.85</v>
+        <v>4588616.59</v>
       </c>
       <c r="P6">
-        <v>18048.23</v>
-      </c>
-      <c r="Q6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B7" t="s">
         <v>25</v>
-      </c>
-      <c r="B7" t="s">
-        <v>26</v>
       </c>
       <c r="C7">
         <v>120041</v>
       </c>
       <c r="D7" t="s">
+        <v>32</v>
+      </c>
+      <c r="E7" t="s">
         <v>33</v>
       </c>
-      <c r="E7" t="s">
-        <v>34</v>
-      </c>
       <c r="F7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G7" t="s">
         <v>21</v>
-      </c>
-      <c r="G7" t="s">
-        <v>22</v>
       </c>
       <c r="H7">
         <v>113750000</v>
       </c>
       <c r="I7">
-        <v>4585072.43</v>
+        <v>18107949.48</v>
       </c>
       <c r="J7">
-        <v>0</v>
+        <v>94161337.299999997</v>
       </c>
       <c r="K7">
-        <v>29802970.760000002</v>
+        <v>82.78</v>
       </c>
       <c r="L7">
-        <v>26.2</v>
+        <v>3621589.9</v>
       </c>
       <c r="M7">
-        <v>1146268.1100000001</v>
+        <v>4554383.3600000003</v>
       </c>
       <c r="N7">
-        <v>4962042.16</v>
+        <v>657172.06000000006</v>
       </c>
       <c r="O7">
-        <v>909080.77</v>
+        <v>4604235.3899999997</v>
       </c>
       <c r="P7">
-        <v>903412.98</v>
-      </c>
-      <c r="Q7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>24</v>
+      </c>
+      <c r="B8" t="s">
         <v>25</v>
-      </c>
-      <c r="B8" t="s">
-        <v>26</v>
       </c>
       <c r="C8">
         <v>105006</v>
       </c>
       <c r="D8" t="s">
+        <v>34</v>
+      </c>
+      <c r="E8" t="s">
         <v>35</v>
       </c>
-      <c r="E8" t="s">
-        <v>36</v>
-      </c>
       <c r="F8" t="s">
+        <v>20</v>
+      </c>
+      <c r="G8" t="s">
         <v>21</v>
-      </c>
-      <c r="G8" t="s">
-        <v>22</v>
       </c>
       <c r="H8">
         <v>39000000</v>
       </c>
       <c r="I8">
-        <v>11216809.310000001</v>
+        <v>29772324.329999998</v>
       </c>
       <c r="J8">
-        <v>0</v>
+        <v>154816086.53</v>
       </c>
       <c r="K8">
-        <v>72909260.519999996</v>
+        <v>396.96</v>
       </c>
       <c r="L8">
-        <v>186.95</v>
+        <v>5954464.8700000001</v>
       </c>
       <c r="M8">
-        <v>2804202.33</v>
+        <v>439413.13</v>
       </c>
       <c r="N8">
-        <v>1262872.3</v>
+        <v>912959.13</v>
       </c>
       <c r="O8">
-        <v>3065018.26</v>
+        <v>5991286.2300000004</v>
       </c>
       <c r="P8">
-        <v>171121.52</v>
-      </c>
-      <c r="Q8">
         <v>0</v>
       </c>
     </row>
@@ -1015,7 +987,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1030,7 +1002,7 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -1048,10 +1020,10 @@
         <v>4</v>
       </c>
       <c r="G1" t="s">
+        <v>37</v>
+      </c>
+      <c r="H1" t="s">
         <v>38</v>
-      </c>
-      <c r="H1" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -1059,25 +1031,25 @@
         <v>105021</v>
       </c>
       <c r="B2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C2" t="s">
         <v>25</v>
-      </c>
-      <c r="C2" t="s">
-        <v>26</v>
       </c>
       <c r="D2">
         <v>105006</v>
       </c>
       <c r="E2" t="s">
+        <v>34</v>
+      </c>
+      <c r="F2" t="s">
         <v>35</v>
       </c>
-      <c r="F2" t="s">
-        <v>36</v>
-      </c>
       <c r="G2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H2">
-        <v>0</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1085,22 +1057,22 @@
         <v>105021</v>
       </c>
       <c r="B3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C3" t="s">
         <v>25</v>
-      </c>
-      <c r="C3" t="s">
-        <v>26</v>
       </c>
       <c r="D3">
         <v>105004</v>
       </c>
       <c r="E3" t="s">
+        <v>30</v>
+      </c>
+      <c r="F3" t="s">
         <v>31</v>
       </c>
-      <c r="F3" t="s">
-        <v>32</v>
-      </c>
       <c r="G3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H3">
         <v>0</v>
@@ -1111,22 +1083,22 @@
         <v>105021</v>
       </c>
       <c r="B4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" t="s">
         <v>25</v>
-      </c>
-      <c r="C4" t="s">
-        <v>26</v>
       </c>
       <c r="D4">
         <v>105003</v>
       </c>
       <c r="E4" t="s">
+        <v>28</v>
+      </c>
+      <c r="F4" t="s">
         <v>29</v>
       </c>
-      <c r="F4" t="s">
-        <v>30</v>
-      </c>
       <c r="G4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H4">
         <v>0</v>
@@ -1137,22 +1109,22 @@
         <v>106002</v>
       </c>
       <c r="B5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" t="s">
         <v>17</v>
-      </c>
-      <c r="C5" t="s">
-        <v>18</v>
       </c>
       <c r="D5">
         <v>120039</v>
       </c>
       <c r="E5" t="s">
+        <v>22</v>
+      </c>
+      <c r="F5" t="s">
         <v>23</v>
       </c>
-      <c r="F5" t="s">
-        <v>24</v>
-      </c>
       <c r="G5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H5">
         <v>0</v>
@@ -1163,22 +1135,22 @@
         <v>106002</v>
       </c>
       <c r="B6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" t="s">
         <v>17</v>
-      </c>
-      <c r="C6" t="s">
-        <v>18</v>
       </c>
       <c r="D6">
         <v>105007</v>
       </c>
       <c r="E6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F6" t="s">
         <v>19</v>
       </c>
-      <c r="F6" t="s">
-        <v>20</v>
-      </c>
       <c r="G6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H6">
         <v>0</v>
@@ -1189,22 +1161,22 @@
         <v>105021</v>
       </c>
       <c r="B7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C7" t="s">
         <v>25</v>
-      </c>
-      <c r="C7" t="s">
-        <v>26</v>
       </c>
       <c r="D7">
         <v>105008</v>
       </c>
       <c r="E7" t="s">
+        <v>26</v>
+      </c>
+      <c r="F7" t="s">
         <v>27</v>
       </c>
-      <c r="F7" t="s">
-        <v>28</v>
-      </c>
       <c r="G7" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H7">
         <v>0</v>
@@ -1215,22 +1187,22 @@
         <v>105021</v>
       </c>
       <c r="B8" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8" t="s">
         <v>25</v>
-      </c>
-      <c r="C8" t="s">
-        <v>26</v>
       </c>
       <c r="D8">
         <v>120041</v>
       </c>
       <c r="E8" t="s">
+        <v>32</v>
+      </c>
+      <c r="F8" t="s">
         <v>33</v>
       </c>
-      <c r="F8" t="s">
-        <v>34</v>
-      </c>
       <c r="G8" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H8">
         <v>0</v>
@@ -1241,25 +1213,25 @@
         <v>105021</v>
       </c>
       <c r="B9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C9" t="s">
         <v>25</v>
-      </c>
-      <c r="C9" t="s">
-        <v>26</v>
       </c>
       <c r="D9">
         <v>105021</v>
       </c>
       <c r="E9" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F9" t="s">
+        <v>40</v>
+      </c>
+      <c r="G9" t="s">
         <v>41</v>
       </c>
-      <c r="G9" t="s">
-        <v>42</v>
-      </c>
       <c r="H9">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -1267,22 +1239,22 @@
         <v>106002</v>
       </c>
       <c r="B10" t="s">
+        <v>16</v>
+      </c>
+      <c r="C10" t="s">
         <v>17</v>
-      </c>
-      <c r="C10" t="s">
-        <v>18</v>
       </c>
       <c r="D10">
         <v>106002</v>
       </c>
       <c r="E10" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F10" t="s">
+        <v>40</v>
+      </c>
+      <c r="G10" t="s">
         <v>41</v>
-      </c>
-      <c r="G10" t="s">
-        <v>42</v>
       </c>
       <c r="H10">
         <v>0</v>

</xml_diff>